<commit_message>
feat: improve timetable quality and teacher leave handling
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="R18768a97c5a84385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="Re8ec417331b5481b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rbfc60f7ccc2e46e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="Rdde3138168cb41c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R47caebb55f8f4a58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R2133225891fb4b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="Rf06b285018d04fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R27a05075d52744e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R07f5a89bfde345f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R1373624dccdd4844"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師勤務" sheetId="11" r:id="R9e0468d652b84b59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R0b6a3dbd4ef84636"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R6d1458f92be64b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="R3abd74077aef4172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R24305d31ddef452c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rffcffd081af14c4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="Rd735f787b77246da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R0dcde41517a84f45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R50c1bea110854274"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="Rb3e66d61ebaa4931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R59a7ee39effa4cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R2d663c8efb2745d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="Rb7d7231c2a2b4799"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R9b158430868a4e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R9501fec8d19f4adf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R76550eaace134a12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28,31 +28,72 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="1">
+  <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF255A83"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8C7D6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8C7D6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8C7D6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C7D6"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -126,6 +167,23 @@
     </x:indexedColors>
   </x:colors>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -348,31 +406,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">時間割入力 v0.1</x:t>
-        </x:is>
+      <x:c r="A1" t="str">
+        <x:v>時間割入力 v0.2</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">IDは表示名と分け、参照にはIDを使用してください。</x:t>
-        </x:is>
+      <x:c r="A2" t="str">
+        <x:v>IDは表示名と分け、参照にはIDを使用してください。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BooleanはExcelのTRUE/FALSE、日付と時刻はExcel型、複数値は半角パイプで入力してください。</x:t>
-        </x:is>
+      <x:c r="A3" t="str">
+        <x:v>BooleanはExcelのTRUE/FALSE、日付と時刻はExcel型、複数値は半角パイプで入力してください。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">配置ルールのin/betweenのcondition_value内部だけは半角スラッシュを使用します。</x:t>
-        </x:is>
+      <x:c r="A4" t="str">
+        <x:v>配置ルールのin/betweenのcondition_value内部だけは半角スラッシュを使用します。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>10_教師休みは、終日休みをALL、時限休みをP1|P2形式で入力します。行がない日時は勤務可能です。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -517,10 +572,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="8.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="9" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="27.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52.220001220703125" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
@@ -528,316 +583,112 @@
     <x:col min="9" max="9" width="3.7799999713897705" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">teacher_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">date</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">period_1_available</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">period_2_available</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">period_3_available</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">period_4_available</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">period_5_available</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">period_6_available</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">note</x:t>
-        </x:is>
-      </x:c>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="7" t="str">
+        <x:v>teacher_id</x:v>
+      </x:c>
+      <x:c r="B1" s="7" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="C1" s="7" t="str">
+        <x:v>unavailable_periods</x:v>
+      </x:c>
+      <x:c r="D1" s="7" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
+      <x:c r="G1"/>
+      <x:c r="H1"/>
+      <x:c r="I1"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="1" t="n">
-        <x:v>46230</x:v>
-      </x:c>
-      <x:c r="C2" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D2" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G2" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H2" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="1" t="n">
-        <x:v>46231</x:v>
-      </x:c>
-      <x:c r="C3" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D3" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E3" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F3" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G3" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H3" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+      <x:c r="H3"/>
+      <x:c r="I3"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="1" t="n">
-        <x:v>46232</x:v>
-      </x:c>
-      <x:c r="C4" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D4" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E4" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F4" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G4" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H4" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A4"/>
+      <x:c r="B4"/>
+      <x:c r="C4"/>
+      <x:c r="D4"/>
+      <x:c r="E4"/>
+      <x:c r="F4"/>
+      <x:c r="G4"/>
+      <x:c r="H4"/>
+      <x:c r="I4"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="1" t="n">
-        <x:v>46233</x:v>
-      </x:c>
-      <x:c r="C5" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D5" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E5" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F5" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G5" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H5" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A5"/>
+      <x:c r="B5"/>
+      <x:c r="C5"/>
+      <x:c r="D5"/>
+      <x:c r="E5"/>
+      <x:c r="F5"/>
+      <x:c r="G5"/>
+      <x:c r="H5"/>
+      <x:c r="I5"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="1" t="n">
-        <x:v>46230</x:v>
-      </x:c>
-      <x:c r="C6" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D6" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E6" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F6" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G6" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H6" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A6"/>
+      <x:c r="B6"/>
+      <x:c r="C6"/>
+      <x:c r="D6"/>
+      <x:c r="E6"/>
+      <x:c r="F6"/>
+      <x:c r="G6"/>
+      <x:c r="H6"/>
+      <x:c r="I6"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="1" t="n">
-        <x:v>46231</x:v>
-      </x:c>
-      <x:c r="C7" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D7" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E7" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F7" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G7" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H7" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A7"/>
+      <x:c r="B7"/>
+      <x:c r="C7"/>
+      <x:c r="D7"/>
+      <x:c r="E7"/>
+      <x:c r="F7"/>
+      <x:c r="G7"/>
+      <x:c r="H7"/>
+      <x:c r="I7"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="1" t="n">
-        <x:v>46232</x:v>
-      </x:c>
-      <x:c r="C8" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D8" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F8" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G8" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H8" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A8"/>
+      <x:c r="B8"/>
+      <x:c r="C8"/>
+      <x:c r="D8"/>
+      <x:c r="E8"/>
+      <x:c r="F8"/>
+      <x:c r="G8"/>
+      <x:c r="H8"/>
+      <x:c r="I8"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="1" t="n">
-        <x:v>46233</x:v>
-      </x:c>
-      <x:c r="C9" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D9" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E9" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F9" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G9" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H9" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A9"/>
+      <x:c r="B9"/>
+      <x:c r="C9"/>
+      <x:c r="D9"/>
+      <x:c r="E9"/>
+      <x:c r="F9"/>
+      <x:c r="G9"/>
+      <x:c r="H9"/>
+      <x:c r="I9"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1348,71 +1199,47 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">setting_key</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">setting_value</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">description</x:t>
-        </x:is>
+      <x:c r="A1" t="str">
+        <x:v>setting_key</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>setting_value</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>description</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">schema_version</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0.1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">入力契約バージョン</x:t>
-        </x:is>
+      <x:c r="A2" t="str">
+        <x:v>schema_version</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>入力契約バージョン</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">timetable_name</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026年度サンプル時間割</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">サンプル</x:t>
-        </x:is>
+      <x:c r="A3" t="str">
+        <x:v>timetable_name</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>2026年度サンプル時間割</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>サンプル</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">description</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">入出力契約v0.1 End-to-End確認用</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">任意</x:t>
-        </x:is>
+      <x:c r="A4" t="str">
+        <x:v>description</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>入出力契約v0.2 End-to-End確認用</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>任意</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2008,71 +1835,57 @@
   <x:cols>
     <x:col min="1" max="1" width="8.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="10.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="3.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">teacher_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">teacher_name</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">enabled</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">note</x:t>
-        </x:is>
+      <x:c r="A1" t="str">
+        <x:v>teacher_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>teacher_name</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>home_campus_id</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">教師一</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A2" t="str">
+        <x:v>T1</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>教師一</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>C1</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">T2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">教師二</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A3" t="str">
+        <x:v>T2</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>教師二</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>C2</x:v>
+      </x:c>
+      <x:c r="D3" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E3"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add lesson count rules and schedule balancing
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,19 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="R3abd74077aef4172"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R24305d31ddef452c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rffcffd081af14c4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="Rd735f787b77246da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R0dcde41517a84f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R50c1bea110854274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="Rb3e66d61ebaa4931"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R59a7ee39effa4cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R2d663c8efb2745d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="Rb7d7231c2a2b4799"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R9b158430868a4e23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R9501fec8d19f4adf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R76550eaace134a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rd0c863f0018b4aa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R75d027d23e1844c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rc5106d69725c4a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R20ac50d698034e5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R01dd08628b3b445a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R30765c53de314763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="Rbaf0a3b82124449d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R80456e69e61d4145"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R449861165fb64b5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R4f7bdfd48bbd4ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R44dea3b5094e430c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R2199bd957bb7446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Rfeb0b0251df6466d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Rab0c124e1ea844ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -41,7 +42,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -53,8 +54,18 @@
         <x:fgColor rgb="FF255A83"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -70,11 +81,25 @@
         <x:color rgb="FFB8C7D6"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -93,6 +118,25 @@
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
         </x:ext>
       </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -184,6 +228,25 @@
     </xfpb:a>
   </xfpb:bag>
 </xfpb:FeaturePropertyBags>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LessonCountRulesTable" displayName="LessonCountRulesTable" ref="A1:K2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="rule_id"/>
+    <x:tableColumn id="2" name="segment_id"/>
+    <x:tableColumn id="3" name="rule_name"/>
+    <x:tableColumn id="4" name="enabled"/>
+    <x:tableColumn id="5" name="class_id"/>
+    <x:tableColumn id="6" name="subject_id"/>
+    <x:tableColumn id="7" name="exact_periods"/>
+    <x:tableColumn id="8" name="start_date"/>
+    <x:tableColumn id="9" name="end_date"/>
+    <x:tableColumn id="10" name="target_periods"/>
+    <x:tableColumn id="11" name="note"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -407,7 +470,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>時間割入力 v0.2</x:v>
+        <x:v>時間割入力 v0.4</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1189,6 +1252,87 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="44" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>rule_id</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>segment_id</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>rule_name</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>class_id</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>subject_id</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>exact_periods</x:v>
+      </x:c>
+      <x:c r="H1" s="13" t="str">
+        <x:v>start_date</x:v>
+      </x:c>
+      <x:c r="I1" s="13" t="str">
+        <x:v>end_date</x:v>
+      </x:c>
+      <x:c r="J1" s="13" t="str">
+        <x:v>target_periods</x:v>
+      </x:c>
+      <x:c r="K1" s="13" t="str">
+        <x:v>note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="16"/>
+      <x:c r="B2" s="16"/>
+      <x:c r="C2" s="16"/>
+      <x:c r="D2" s="16"/>
+      <x:c r="E2" s="16"/>
+      <x:c r="F2" s="16"/>
+      <x:c r="G2" s="16"/>
+      <x:c r="H2" s="17"/>
+      <x:c r="I2" s="17"/>
+      <x:c r="J2" s="16"/>
+      <x:c r="K2" s="16"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="D2:D1000">
+      <x:formula1>"true,false"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="whole" sqref="G2:G1000">
+      <x:formula1>0</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b72c863e81c483a"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1214,7 +1358,7 @@
         <x:v>schema_version</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>0.3</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>入力契約バージョン</x:v>

</xml_diff>

<commit_message>
Add rules and warm-start timetable solver
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,20 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rd0c863f0018b4aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R75d027d23e1844c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rc5106d69725c4a39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R20ac50d698034e5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R01dd08628b3b445a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R30765c53de314763"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="Rbaf0a3b82124449d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R80456e69e61d4145"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R449861165fb64b5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R4f7bdfd48bbd4ed6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R44dea3b5094e430c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R2199bd957bb7446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Rfeb0b0251df6466d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Rab0c124e1ea844ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rce4ae57acdfb44a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R0308edaba3fb495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R7a74fc55705a42ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R5596ec139a5f40c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Re87ea8e2795b4752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R1ac5bae294f74ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R2efc711d8d0a4be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R73be8cafad4d4c48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R1a287a622e884461"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R264f9bb3df35474e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R3d040cf4870b4dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R7ed81da29cae4872"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R3d27d55fe55c43b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="R333f07f4aa704b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Rcd0b11a2534e4cd9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,7 +43,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -52,6 +53,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF255A83"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -99,7 +110,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -137,6 +148,23 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -780,6 +808,7 @@
     <x:col min="16" max="16" width="17.780000686645508" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="5.559999942779541" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="3.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="31" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -873,6 +902,9 @@
           <x:t xml:space="preserve">note</x:t>
         </x:is>
       </x:c>
+      <x:c r="S1" t="str">
+        <x:v>preferred_attendance_streak_limit</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="inlineStr">
@@ -946,9 +978,7 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="P2" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="P2"/>
       <x:c r="Q2" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -1032,11 +1062,7 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="P3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="P3"/>
       <x:c r="Q3" t="n">
         <x:v>20</x:v>
       </x:c>
@@ -1114,9 +1140,7 @@
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="P4" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="P4"/>
       <x:c r="Q4" t="n">
         <x:v>30</x:v>
       </x:c>
@@ -1208,6 +1232,94 @@
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>RULE_ATTENDANCE_EXAM</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>受験学年の連続登校選好</x:v>
+      </x:c>
+      <x:c r="C6" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>hard</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>class</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>exam_category</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>eq</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>exam</x:v>
+      </x:c>
+      <x:c r="I6"/>
+      <x:c r="J6"/>
+      <x:c r="K6"/>
+      <x:c r="L6"/>
+      <x:c r="M6"/>
+      <x:c r="N6"/>
+      <x:c r="O6"/>
+      <x:c r="P6"/>
+      <x:c r="Q6" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R6" t="str">
+        <x:v>S18: 3日まで無罰、4日目以降を段階的に抑制</x:v>
+      </x:c>
+      <x:c r="S6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>RULE_ATTENDANCE_NON_EXAM</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>非受験学年の連続登校制御</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>hard</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>class</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>exam_category</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>in</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>non_exam/special/none</x:v>
+      </x:c>
+      <x:c r="I7"/>
+      <x:c r="J7"/>
+      <x:c r="K7"/>
+      <x:c r="L7"/>
+      <x:c r="M7"/>
+      <x:c r="N7"/>
+      <x:c r="O7"/>
+      <x:c r="P7" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="Q7" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="R7" t="str">
+        <x:v>H10: 4日以上禁止、S18: 3日連続を軽く抑制</x:v>
+      </x:c>
+      <x:c r="S7" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1328,8 +1440,1092 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b72c863e81c483a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R282735b136654e9a"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="47.779998779296875" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="33.33000183105469" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="13.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="46.66999816894531" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="25.5" customHeight="1">
+      <x:c r="A1" s="23" t="str">
+        <x:v>rule_id</x:v>
+      </x:c>
+      <x:c r="B1" s="23" t="str">
+        <x:v>segment_id</x:v>
+      </x:c>
+      <x:c r="C1" s="23" t="str">
+        <x:v>rule_name</x:v>
+      </x:c>
+      <x:c r="D1" s="23" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="E1" s="23" t="str">
+        <x:v>class_id</x:v>
+      </x:c>
+      <x:c r="F1" s="23" t="str">
+        <x:v>subject_id</x:v>
+      </x:c>
+      <x:c r="G1" s="23" t="str">
+        <x:v>preferred_periods</x:v>
+      </x:c>
+      <x:c r="H1" s="23" t="str">
+        <x:v>start_date</x:v>
+      </x:c>
+      <x:c r="I1" s="23" t="str">
+        <x:v>end_date</x:v>
+      </x:c>
+      <x:c r="J1" s="23" t="str">
+        <x:v>target_periods</x:v>
+      </x:c>
+      <x:c r="K1" s="23" t="str">
+        <x:v>note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="26"/>
+      <x:c r="B2" s="26"/>
+      <x:c r="C2" s="26"/>
+      <x:c r="D2" s="26"/>
+      <x:c r="E2" s="26"/>
+      <x:c r="F2" s="26"/>
+      <x:c r="G2" s="26"/>
+      <x:c r="H2" s="26"/>
+      <x:c r="I2" s="26"/>
+      <x:c r="J2" s="26"/>
+      <x:c r="K2" s="26"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="26"/>
+      <x:c r="B3" s="26"/>
+      <x:c r="C3" s="26"/>
+      <x:c r="D3" s="26"/>
+      <x:c r="E3" s="26"/>
+      <x:c r="F3" s="26"/>
+      <x:c r="G3" s="26"/>
+      <x:c r="H3" s="26"/>
+      <x:c r="I3" s="26"/>
+      <x:c r="J3" s="26"/>
+      <x:c r="K3" s="26"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="26"/>
+      <x:c r="B4" s="26"/>
+      <x:c r="C4" s="26"/>
+      <x:c r="D4" s="26"/>
+      <x:c r="E4" s="26"/>
+      <x:c r="F4" s="26"/>
+      <x:c r="G4" s="26"/>
+      <x:c r="H4" s="26"/>
+      <x:c r="I4" s="26"/>
+      <x:c r="J4" s="26"/>
+      <x:c r="K4" s="26"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="26"/>
+      <x:c r="B5" s="26"/>
+      <x:c r="C5" s="26"/>
+      <x:c r="D5" s="26"/>
+      <x:c r="E5" s="26"/>
+      <x:c r="F5" s="26"/>
+      <x:c r="G5" s="26"/>
+      <x:c r="H5" s="26"/>
+      <x:c r="I5" s="26"/>
+      <x:c r="J5" s="26"/>
+      <x:c r="K5" s="26"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="26"/>
+      <x:c r="B6" s="26"/>
+      <x:c r="C6" s="26"/>
+      <x:c r="D6" s="26"/>
+      <x:c r="E6" s="26"/>
+      <x:c r="F6" s="26"/>
+      <x:c r="G6" s="26"/>
+      <x:c r="H6" s="26"/>
+      <x:c r="I6" s="26"/>
+      <x:c r="J6" s="26"/>
+      <x:c r="K6" s="26"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="26"/>
+      <x:c r="B7" s="26"/>
+      <x:c r="C7" s="26"/>
+      <x:c r="D7" s="26"/>
+      <x:c r="E7" s="26"/>
+      <x:c r="F7" s="26"/>
+      <x:c r="G7" s="26"/>
+      <x:c r="H7" s="26"/>
+      <x:c r="I7" s="26"/>
+      <x:c r="J7" s="26"/>
+      <x:c r="K7" s="26"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="26"/>
+      <x:c r="B8" s="26"/>
+      <x:c r="C8" s="26"/>
+      <x:c r="D8" s="26"/>
+      <x:c r="E8" s="26"/>
+      <x:c r="F8" s="26"/>
+      <x:c r="G8" s="26"/>
+      <x:c r="H8" s="26"/>
+      <x:c r="I8" s="26"/>
+      <x:c r="J8" s="26"/>
+      <x:c r="K8" s="26"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="26"/>
+      <x:c r="B9" s="26"/>
+      <x:c r="C9" s="26"/>
+      <x:c r="D9" s="26"/>
+      <x:c r="E9" s="26"/>
+      <x:c r="F9" s="26"/>
+      <x:c r="G9" s="26"/>
+      <x:c r="H9" s="26"/>
+      <x:c r="I9" s="26"/>
+      <x:c r="J9" s="26"/>
+      <x:c r="K9" s="26"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="26"/>
+      <x:c r="B10" s="26"/>
+      <x:c r="C10" s="26"/>
+      <x:c r="D10" s="26"/>
+      <x:c r="E10" s="26"/>
+      <x:c r="F10" s="26"/>
+      <x:c r="G10" s="26"/>
+      <x:c r="H10" s="26"/>
+      <x:c r="I10" s="26"/>
+      <x:c r="J10" s="26"/>
+      <x:c r="K10" s="26"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="26"/>
+      <x:c r="B11" s="26"/>
+      <x:c r="C11" s="26"/>
+      <x:c r="D11" s="26"/>
+      <x:c r="E11" s="26"/>
+      <x:c r="F11" s="26"/>
+      <x:c r="G11" s="26"/>
+      <x:c r="H11" s="26"/>
+      <x:c r="I11" s="26"/>
+      <x:c r="J11" s="26"/>
+      <x:c r="K11" s="26"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="26"/>
+      <x:c r="B12" s="26"/>
+      <x:c r="C12" s="26"/>
+      <x:c r="D12" s="26"/>
+      <x:c r="E12" s="26"/>
+      <x:c r="F12" s="26"/>
+      <x:c r="G12" s="26"/>
+      <x:c r="H12" s="26"/>
+      <x:c r="I12" s="26"/>
+      <x:c r="J12" s="26"/>
+      <x:c r="K12" s="26"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="26"/>
+      <x:c r="B13" s="26"/>
+      <x:c r="C13" s="26"/>
+      <x:c r="D13" s="26"/>
+      <x:c r="E13" s="26"/>
+      <x:c r="F13" s="26"/>
+      <x:c r="G13" s="26"/>
+      <x:c r="H13" s="26"/>
+      <x:c r="I13" s="26"/>
+      <x:c r="J13" s="26"/>
+      <x:c r="K13" s="26"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="26"/>
+      <x:c r="B14" s="26"/>
+      <x:c r="C14" s="26"/>
+      <x:c r="D14" s="26"/>
+      <x:c r="E14" s="26"/>
+      <x:c r="F14" s="26"/>
+      <x:c r="G14" s="26"/>
+      <x:c r="H14" s="26"/>
+      <x:c r="I14" s="26"/>
+      <x:c r="J14" s="26"/>
+      <x:c r="K14" s="26"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="26"/>
+      <x:c r="B15" s="26"/>
+      <x:c r="C15" s="26"/>
+      <x:c r="D15" s="26"/>
+      <x:c r="E15" s="26"/>
+      <x:c r="F15" s="26"/>
+      <x:c r="G15" s="26"/>
+      <x:c r="H15" s="26"/>
+      <x:c r="I15" s="26"/>
+      <x:c r="J15" s="26"/>
+      <x:c r="K15" s="26"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="26"/>
+      <x:c r="B16" s="26"/>
+      <x:c r="C16" s="26"/>
+      <x:c r="D16" s="26"/>
+      <x:c r="E16" s="26"/>
+      <x:c r="F16" s="26"/>
+      <x:c r="G16" s="26"/>
+      <x:c r="H16" s="26"/>
+      <x:c r="I16" s="26"/>
+      <x:c r="J16" s="26"/>
+      <x:c r="K16" s="26"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="26"/>
+      <x:c r="B17" s="26"/>
+      <x:c r="C17" s="26"/>
+      <x:c r="D17" s="26"/>
+      <x:c r="E17" s="26"/>
+      <x:c r="F17" s="26"/>
+      <x:c r="G17" s="26"/>
+      <x:c r="H17" s="26"/>
+      <x:c r="I17" s="26"/>
+      <x:c r="J17" s="26"/>
+      <x:c r="K17" s="26"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="26"/>
+      <x:c r="B18" s="26"/>
+      <x:c r="C18" s="26"/>
+      <x:c r="D18" s="26"/>
+      <x:c r="E18" s="26"/>
+      <x:c r="F18" s="26"/>
+      <x:c r="G18" s="26"/>
+      <x:c r="H18" s="26"/>
+      <x:c r="I18" s="26"/>
+      <x:c r="J18" s="26"/>
+      <x:c r="K18" s="26"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="26"/>
+      <x:c r="B19" s="26"/>
+      <x:c r="C19" s="26"/>
+      <x:c r="D19" s="26"/>
+      <x:c r="E19" s="26"/>
+      <x:c r="F19" s="26"/>
+      <x:c r="G19" s="26"/>
+      <x:c r="H19" s="26"/>
+      <x:c r="I19" s="26"/>
+      <x:c r="J19" s="26"/>
+      <x:c r="K19" s="26"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="26"/>
+      <x:c r="B20" s="26"/>
+      <x:c r="C20" s="26"/>
+      <x:c r="D20" s="26"/>
+      <x:c r="E20" s="26"/>
+      <x:c r="F20" s="26"/>
+      <x:c r="G20" s="26"/>
+      <x:c r="H20" s="26"/>
+      <x:c r="I20" s="26"/>
+      <x:c r="J20" s="26"/>
+      <x:c r="K20" s="26"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="26"/>
+      <x:c r="B21" s="26"/>
+      <x:c r="C21" s="26"/>
+      <x:c r="D21" s="26"/>
+      <x:c r="E21" s="26"/>
+      <x:c r="F21" s="26"/>
+      <x:c r="G21" s="26"/>
+      <x:c r="H21" s="26"/>
+      <x:c r="I21" s="26"/>
+      <x:c r="J21" s="26"/>
+      <x:c r="K21" s="26"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="26"/>
+      <x:c r="B22" s="26"/>
+      <x:c r="C22" s="26"/>
+      <x:c r="D22" s="26"/>
+      <x:c r="E22" s="26"/>
+      <x:c r="F22" s="26"/>
+      <x:c r="G22" s="26"/>
+      <x:c r="H22" s="26"/>
+      <x:c r="I22" s="26"/>
+      <x:c r="J22" s="26"/>
+      <x:c r="K22" s="26"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="26"/>
+      <x:c r="B23" s="26"/>
+      <x:c r="C23" s="26"/>
+      <x:c r="D23" s="26"/>
+      <x:c r="E23" s="26"/>
+      <x:c r="F23" s="26"/>
+      <x:c r="G23" s="26"/>
+      <x:c r="H23" s="26"/>
+      <x:c r="I23" s="26"/>
+      <x:c r="J23" s="26"/>
+      <x:c r="K23" s="26"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="26"/>
+      <x:c r="B24" s="26"/>
+      <x:c r="C24" s="26"/>
+      <x:c r="D24" s="26"/>
+      <x:c r="E24" s="26"/>
+      <x:c r="F24" s="26"/>
+      <x:c r="G24" s="26"/>
+      <x:c r="H24" s="26"/>
+      <x:c r="I24" s="26"/>
+      <x:c r="J24" s="26"/>
+      <x:c r="K24" s="26"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="26"/>
+      <x:c r="B25" s="26"/>
+      <x:c r="C25" s="26"/>
+      <x:c r="D25" s="26"/>
+      <x:c r="E25" s="26"/>
+      <x:c r="F25" s="26"/>
+      <x:c r="G25" s="26"/>
+      <x:c r="H25" s="26"/>
+      <x:c r="I25" s="26"/>
+      <x:c r="J25" s="26"/>
+      <x:c r="K25" s="26"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="26"/>
+      <x:c r="B26" s="26"/>
+      <x:c r="C26" s="26"/>
+      <x:c r="D26" s="26"/>
+      <x:c r="E26" s="26"/>
+      <x:c r="F26" s="26"/>
+      <x:c r="G26" s="26"/>
+      <x:c r="H26" s="26"/>
+      <x:c r="I26" s="26"/>
+      <x:c r="J26" s="26"/>
+      <x:c r="K26" s="26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="26"/>
+      <x:c r="B27" s="26"/>
+      <x:c r="C27" s="26"/>
+      <x:c r="D27" s="26"/>
+      <x:c r="E27" s="26"/>
+      <x:c r="F27" s="26"/>
+      <x:c r="G27" s="26"/>
+      <x:c r="H27" s="26"/>
+      <x:c r="I27" s="26"/>
+      <x:c r="J27" s="26"/>
+      <x:c r="K27" s="26"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="26"/>
+      <x:c r="B28" s="26"/>
+      <x:c r="C28" s="26"/>
+      <x:c r="D28" s="26"/>
+      <x:c r="E28" s="26"/>
+      <x:c r="F28" s="26"/>
+      <x:c r="G28" s="26"/>
+      <x:c r="H28" s="26"/>
+      <x:c r="I28" s="26"/>
+      <x:c r="J28" s="26"/>
+      <x:c r="K28" s="26"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="26"/>
+      <x:c r="B29" s="26"/>
+      <x:c r="C29" s="26"/>
+      <x:c r="D29" s="26"/>
+      <x:c r="E29" s="26"/>
+      <x:c r="F29" s="26"/>
+      <x:c r="G29" s="26"/>
+      <x:c r="H29" s="26"/>
+      <x:c r="I29" s="26"/>
+      <x:c r="J29" s="26"/>
+      <x:c r="K29" s="26"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="26"/>
+      <x:c r="B30" s="26"/>
+      <x:c r="C30" s="26"/>
+      <x:c r="D30" s="26"/>
+      <x:c r="E30" s="26"/>
+      <x:c r="F30" s="26"/>
+      <x:c r="G30" s="26"/>
+      <x:c r="H30" s="26"/>
+      <x:c r="I30" s="26"/>
+      <x:c r="J30" s="26"/>
+      <x:c r="K30" s="26"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="26"/>
+      <x:c r="B31" s="26"/>
+      <x:c r="C31" s="26"/>
+      <x:c r="D31" s="26"/>
+      <x:c r="E31" s="26"/>
+      <x:c r="F31" s="26"/>
+      <x:c r="G31" s="26"/>
+      <x:c r="H31" s="26"/>
+      <x:c r="I31" s="26"/>
+      <x:c r="J31" s="26"/>
+      <x:c r="K31" s="26"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="26"/>
+      <x:c r="B32" s="26"/>
+      <x:c r="C32" s="26"/>
+      <x:c r="D32" s="26"/>
+      <x:c r="E32" s="26"/>
+      <x:c r="F32" s="26"/>
+      <x:c r="G32" s="26"/>
+      <x:c r="H32" s="26"/>
+      <x:c r="I32" s="26"/>
+      <x:c r="J32" s="26"/>
+      <x:c r="K32" s="26"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="26"/>
+      <x:c r="B33" s="26"/>
+      <x:c r="C33" s="26"/>
+      <x:c r="D33" s="26"/>
+      <x:c r="E33" s="26"/>
+      <x:c r="F33" s="26"/>
+      <x:c r="G33" s="26"/>
+      <x:c r="H33" s="26"/>
+      <x:c r="I33" s="26"/>
+      <x:c r="J33" s="26"/>
+      <x:c r="K33" s="26"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="26"/>
+      <x:c r="B34" s="26"/>
+      <x:c r="C34" s="26"/>
+      <x:c r="D34" s="26"/>
+      <x:c r="E34" s="26"/>
+      <x:c r="F34" s="26"/>
+      <x:c r="G34" s="26"/>
+      <x:c r="H34" s="26"/>
+      <x:c r="I34" s="26"/>
+      <x:c r="J34" s="26"/>
+      <x:c r="K34" s="26"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="26"/>
+      <x:c r="B35" s="26"/>
+      <x:c r="C35" s="26"/>
+      <x:c r="D35" s="26"/>
+      <x:c r="E35" s="26"/>
+      <x:c r="F35" s="26"/>
+      <x:c r="G35" s="26"/>
+      <x:c r="H35" s="26"/>
+      <x:c r="I35" s="26"/>
+      <x:c r="J35" s="26"/>
+      <x:c r="K35" s="26"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="26"/>
+      <x:c r="B36" s="26"/>
+      <x:c r="C36" s="26"/>
+      <x:c r="D36" s="26"/>
+      <x:c r="E36" s="26"/>
+      <x:c r="F36" s="26"/>
+      <x:c r="G36" s="26"/>
+      <x:c r="H36" s="26"/>
+      <x:c r="I36" s="26"/>
+      <x:c r="J36" s="26"/>
+      <x:c r="K36" s="26"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="26"/>
+      <x:c r="B37" s="26"/>
+      <x:c r="C37" s="26"/>
+      <x:c r="D37" s="26"/>
+      <x:c r="E37" s="26"/>
+      <x:c r="F37" s="26"/>
+      <x:c r="G37" s="26"/>
+      <x:c r="H37" s="26"/>
+      <x:c r="I37" s="26"/>
+      <x:c r="J37" s="26"/>
+      <x:c r="K37" s="26"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="26"/>
+      <x:c r="B38" s="26"/>
+      <x:c r="C38" s="26"/>
+      <x:c r="D38" s="26"/>
+      <x:c r="E38" s="26"/>
+      <x:c r="F38" s="26"/>
+      <x:c r="G38" s="26"/>
+      <x:c r="H38" s="26"/>
+      <x:c r="I38" s="26"/>
+      <x:c r="J38" s="26"/>
+      <x:c r="K38" s="26"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="26"/>
+      <x:c r="B39" s="26"/>
+      <x:c r="C39" s="26"/>
+      <x:c r="D39" s="26"/>
+      <x:c r="E39" s="26"/>
+      <x:c r="F39" s="26"/>
+      <x:c r="G39" s="26"/>
+      <x:c r="H39" s="26"/>
+      <x:c r="I39" s="26"/>
+      <x:c r="J39" s="26"/>
+      <x:c r="K39" s="26"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="26"/>
+      <x:c r="B40" s="26"/>
+      <x:c r="C40" s="26"/>
+      <x:c r="D40" s="26"/>
+      <x:c r="E40" s="26"/>
+      <x:c r="F40" s="26"/>
+      <x:c r="G40" s="26"/>
+      <x:c r="H40" s="26"/>
+      <x:c r="I40" s="26"/>
+      <x:c r="J40" s="26"/>
+      <x:c r="K40" s="26"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="26"/>
+      <x:c r="B41" s="26"/>
+      <x:c r="C41" s="26"/>
+      <x:c r="D41" s="26"/>
+      <x:c r="E41" s="26"/>
+      <x:c r="F41" s="26"/>
+      <x:c r="G41" s="26"/>
+      <x:c r="H41" s="26"/>
+      <x:c r="I41" s="26"/>
+      <x:c r="J41" s="26"/>
+      <x:c r="K41" s="26"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="26"/>
+      <x:c r="B42" s="26"/>
+      <x:c r="C42" s="26"/>
+      <x:c r="D42" s="26"/>
+      <x:c r="E42" s="26"/>
+      <x:c r="F42" s="26"/>
+      <x:c r="G42" s="26"/>
+      <x:c r="H42" s="26"/>
+      <x:c r="I42" s="26"/>
+      <x:c r="J42" s="26"/>
+      <x:c r="K42" s="26"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="26"/>
+      <x:c r="B43" s="26"/>
+      <x:c r="C43" s="26"/>
+      <x:c r="D43" s="26"/>
+      <x:c r="E43" s="26"/>
+      <x:c r="F43" s="26"/>
+      <x:c r="G43" s="26"/>
+      <x:c r="H43" s="26"/>
+      <x:c r="I43" s="26"/>
+      <x:c r="J43" s="26"/>
+      <x:c r="K43" s="26"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="26"/>
+      <x:c r="B44" s="26"/>
+      <x:c r="C44" s="26"/>
+      <x:c r="D44" s="26"/>
+      <x:c r="E44" s="26"/>
+      <x:c r="F44" s="26"/>
+      <x:c r="G44" s="26"/>
+      <x:c r="H44" s="26"/>
+      <x:c r="I44" s="26"/>
+      <x:c r="J44" s="26"/>
+      <x:c r="K44" s="26"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="26"/>
+      <x:c r="B45" s="26"/>
+      <x:c r="C45" s="26"/>
+      <x:c r="D45" s="26"/>
+      <x:c r="E45" s="26"/>
+      <x:c r="F45" s="26"/>
+      <x:c r="G45" s="26"/>
+      <x:c r="H45" s="26"/>
+      <x:c r="I45" s="26"/>
+      <x:c r="J45" s="26"/>
+      <x:c r="K45" s="26"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="26"/>
+      <x:c r="B46" s="26"/>
+      <x:c r="C46" s="26"/>
+      <x:c r="D46" s="26"/>
+      <x:c r="E46" s="26"/>
+      <x:c r="F46" s="26"/>
+      <x:c r="G46" s="26"/>
+      <x:c r="H46" s="26"/>
+      <x:c r="I46" s="26"/>
+      <x:c r="J46" s="26"/>
+      <x:c r="K46" s="26"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="26"/>
+      <x:c r="B47" s="26"/>
+      <x:c r="C47" s="26"/>
+      <x:c r="D47" s="26"/>
+      <x:c r="E47" s="26"/>
+      <x:c r="F47" s="26"/>
+      <x:c r="G47" s="26"/>
+      <x:c r="H47" s="26"/>
+      <x:c r="I47" s="26"/>
+      <x:c r="J47" s="26"/>
+      <x:c r="K47" s="26"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="26"/>
+      <x:c r="B48" s="26"/>
+      <x:c r="C48" s="26"/>
+      <x:c r="D48" s="26"/>
+      <x:c r="E48" s="26"/>
+      <x:c r="F48" s="26"/>
+      <x:c r="G48" s="26"/>
+      <x:c r="H48" s="26"/>
+      <x:c r="I48" s="26"/>
+      <x:c r="J48" s="26"/>
+      <x:c r="K48" s="26"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="26"/>
+      <x:c r="B49" s="26"/>
+      <x:c r="C49" s="26"/>
+      <x:c r="D49" s="26"/>
+      <x:c r="E49" s="26"/>
+      <x:c r="F49" s="26"/>
+      <x:c r="G49" s="26"/>
+      <x:c r="H49" s="26"/>
+      <x:c r="I49" s="26"/>
+      <x:c r="J49" s="26"/>
+      <x:c r="K49" s="26"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="26"/>
+      <x:c r="B50" s="26"/>
+      <x:c r="C50" s="26"/>
+      <x:c r="D50" s="26"/>
+      <x:c r="E50" s="26"/>
+      <x:c r="F50" s="26"/>
+      <x:c r="G50" s="26"/>
+      <x:c r="H50" s="26"/>
+      <x:c r="I50" s="26"/>
+      <x:c r="J50" s="26"/>
+      <x:c r="K50" s="26"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="26"/>
+      <x:c r="B51" s="26"/>
+      <x:c r="C51" s="26"/>
+      <x:c r="D51" s="26"/>
+      <x:c r="E51" s="26"/>
+      <x:c r="F51" s="26"/>
+      <x:c r="G51" s="26"/>
+      <x:c r="H51" s="26"/>
+      <x:c r="I51" s="26"/>
+      <x:c r="J51" s="26"/>
+      <x:c r="K51" s="26"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="26"/>
+      <x:c r="B52" s="26"/>
+      <x:c r="C52" s="26"/>
+      <x:c r="D52" s="26"/>
+      <x:c r="E52" s="26"/>
+      <x:c r="F52" s="26"/>
+      <x:c r="G52" s="26"/>
+      <x:c r="H52" s="26"/>
+      <x:c r="I52" s="26"/>
+      <x:c r="J52" s="26"/>
+      <x:c r="K52" s="26"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="26"/>
+      <x:c r="B53" s="26"/>
+      <x:c r="C53" s="26"/>
+      <x:c r="D53" s="26"/>
+      <x:c r="E53" s="26"/>
+      <x:c r="F53" s="26"/>
+      <x:c r="G53" s="26"/>
+      <x:c r="H53" s="26"/>
+      <x:c r="I53" s="26"/>
+      <x:c r="J53" s="26"/>
+      <x:c r="K53" s="26"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="26"/>
+      <x:c r="B54" s="26"/>
+      <x:c r="C54" s="26"/>
+      <x:c r="D54" s="26"/>
+      <x:c r="E54" s="26"/>
+      <x:c r="F54" s="26"/>
+      <x:c r="G54" s="26"/>
+      <x:c r="H54" s="26"/>
+      <x:c r="I54" s="26"/>
+      <x:c r="J54" s="26"/>
+      <x:c r="K54" s="26"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="26"/>
+      <x:c r="B55" s="26"/>
+      <x:c r="C55" s="26"/>
+      <x:c r="D55" s="26"/>
+      <x:c r="E55" s="26"/>
+      <x:c r="F55" s="26"/>
+      <x:c r="G55" s="26"/>
+      <x:c r="H55" s="26"/>
+      <x:c r="I55" s="26"/>
+      <x:c r="J55" s="26"/>
+      <x:c r="K55" s="26"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="26"/>
+      <x:c r="B56" s="26"/>
+      <x:c r="C56" s="26"/>
+      <x:c r="D56" s="26"/>
+      <x:c r="E56" s="26"/>
+      <x:c r="F56" s="26"/>
+      <x:c r="G56" s="26"/>
+      <x:c r="H56" s="26"/>
+      <x:c r="I56" s="26"/>
+      <x:c r="J56" s="26"/>
+      <x:c r="K56" s="26"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="26"/>
+      <x:c r="B57" s="26"/>
+      <x:c r="C57" s="26"/>
+      <x:c r="D57" s="26"/>
+      <x:c r="E57" s="26"/>
+      <x:c r="F57" s="26"/>
+      <x:c r="G57" s="26"/>
+      <x:c r="H57" s="26"/>
+      <x:c r="I57" s="26"/>
+      <x:c r="J57" s="26"/>
+      <x:c r="K57" s="26"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="26"/>
+      <x:c r="B58" s="26"/>
+      <x:c r="C58" s="26"/>
+      <x:c r="D58" s="26"/>
+      <x:c r="E58" s="26"/>
+      <x:c r="F58" s="26"/>
+      <x:c r="G58" s="26"/>
+      <x:c r="H58" s="26"/>
+      <x:c r="I58" s="26"/>
+      <x:c r="J58" s="26"/>
+      <x:c r="K58" s="26"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="26"/>
+      <x:c r="B59" s="26"/>
+      <x:c r="C59" s="26"/>
+      <x:c r="D59" s="26"/>
+      <x:c r="E59" s="26"/>
+      <x:c r="F59" s="26"/>
+      <x:c r="G59" s="26"/>
+      <x:c r="H59" s="26"/>
+      <x:c r="I59" s="26"/>
+      <x:c r="J59" s="26"/>
+      <x:c r="K59" s="26"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="26"/>
+      <x:c r="B60" s="26"/>
+      <x:c r="C60" s="26"/>
+      <x:c r="D60" s="26"/>
+      <x:c r="E60" s="26"/>
+      <x:c r="F60" s="26"/>
+      <x:c r="G60" s="26"/>
+      <x:c r="H60" s="26"/>
+      <x:c r="I60" s="26"/>
+      <x:c r="J60" s="26"/>
+      <x:c r="K60" s="26"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="26"/>
+      <x:c r="B61" s="26"/>
+      <x:c r="C61" s="26"/>
+      <x:c r="D61" s="26"/>
+      <x:c r="E61" s="26"/>
+      <x:c r="F61" s="26"/>
+      <x:c r="G61" s="26"/>
+      <x:c r="H61" s="26"/>
+      <x:c r="I61" s="26"/>
+      <x:c r="J61" s="26"/>
+      <x:c r="K61" s="26"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="26"/>
+      <x:c r="B62" s="26"/>
+      <x:c r="C62" s="26"/>
+      <x:c r="D62" s="26"/>
+      <x:c r="E62" s="26"/>
+      <x:c r="F62" s="26"/>
+      <x:c r="G62" s="26"/>
+      <x:c r="H62" s="26"/>
+      <x:c r="I62" s="26"/>
+      <x:c r="J62" s="26"/>
+      <x:c r="K62" s="26"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="26"/>
+      <x:c r="B63" s="26"/>
+      <x:c r="C63" s="26"/>
+      <x:c r="D63" s="26"/>
+      <x:c r="E63" s="26"/>
+      <x:c r="F63" s="26"/>
+      <x:c r="G63" s="26"/>
+      <x:c r="H63" s="26"/>
+      <x:c r="I63" s="26"/>
+      <x:c r="J63" s="26"/>
+      <x:c r="K63" s="26"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="26"/>
+      <x:c r="B64" s="26"/>
+      <x:c r="C64" s="26"/>
+      <x:c r="D64" s="26"/>
+      <x:c r="E64" s="26"/>
+      <x:c r="F64" s="26"/>
+      <x:c r="G64" s="26"/>
+      <x:c r="H64" s="26"/>
+      <x:c r="I64" s="26"/>
+      <x:c r="J64" s="26"/>
+      <x:c r="K64" s="26"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="26"/>
+      <x:c r="B65" s="26"/>
+      <x:c r="C65" s="26"/>
+      <x:c r="D65" s="26"/>
+      <x:c r="E65" s="26"/>
+      <x:c r="F65" s="26"/>
+      <x:c r="G65" s="26"/>
+      <x:c r="H65" s="26"/>
+      <x:c r="I65" s="26"/>
+      <x:c r="J65" s="26"/>
+      <x:c r="K65" s="26"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="26"/>
+      <x:c r="B66" s="26"/>
+      <x:c r="C66" s="26"/>
+      <x:c r="D66" s="26"/>
+      <x:c r="E66" s="26"/>
+      <x:c r="F66" s="26"/>
+      <x:c r="G66" s="26"/>
+      <x:c r="H66" s="26"/>
+      <x:c r="I66" s="26"/>
+      <x:c r="J66" s="26"/>
+      <x:c r="K66" s="26"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="26"/>
+      <x:c r="B67" s="26"/>
+      <x:c r="C67" s="26"/>
+      <x:c r="D67" s="26"/>
+      <x:c r="E67" s="26"/>
+      <x:c r="F67" s="26"/>
+      <x:c r="G67" s="26"/>
+      <x:c r="H67" s="26"/>
+      <x:c r="I67" s="26"/>
+      <x:c r="J67" s="26"/>
+      <x:c r="K67" s="26"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="26"/>
+      <x:c r="B68" s="26"/>
+      <x:c r="C68" s="26"/>
+      <x:c r="D68" s="26"/>
+      <x:c r="E68" s="26"/>
+      <x:c r="F68" s="26"/>
+      <x:c r="G68" s="26"/>
+      <x:c r="H68" s="26"/>
+      <x:c r="I68" s="26"/>
+      <x:c r="J68" s="26"/>
+      <x:c r="K68" s="26"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="26"/>
+      <x:c r="B69" s="26"/>
+      <x:c r="C69" s="26"/>
+      <x:c r="D69" s="26"/>
+      <x:c r="E69" s="26"/>
+      <x:c r="F69" s="26"/>
+      <x:c r="G69" s="26"/>
+      <x:c r="H69" s="26"/>
+      <x:c r="I69" s="26"/>
+      <x:c r="J69" s="26"/>
+      <x:c r="K69" s="26"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="26"/>
+      <x:c r="B70" s="26"/>
+      <x:c r="C70" s="26"/>
+      <x:c r="D70" s="26"/>
+      <x:c r="E70" s="26"/>
+      <x:c r="F70" s="26"/>
+      <x:c r="G70" s="26"/>
+      <x:c r="H70" s="26"/>
+      <x:c r="I70" s="26"/>
+      <x:c r="J70" s="26"/>
+      <x:c r="K70" s="26"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="26"/>
+      <x:c r="B71" s="26"/>
+      <x:c r="C71" s="26"/>
+      <x:c r="D71" s="26"/>
+      <x:c r="E71" s="26"/>
+      <x:c r="F71" s="26"/>
+      <x:c r="G71" s="26"/>
+      <x:c r="H71" s="26"/>
+      <x:c r="I71" s="26"/>
+      <x:c r="J71" s="26"/>
+      <x:c r="K71" s="26"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="26"/>
+      <x:c r="B72" s="26"/>
+      <x:c r="C72" s="26"/>
+      <x:c r="D72" s="26"/>
+      <x:c r="E72" s="26"/>
+      <x:c r="F72" s="26"/>
+      <x:c r="G72" s="26"/>
+      <x:c r="H72" s="26"/>
+      <x:c r="I72" s="26"/>
+      <x:c r="J72" s="26"/>
+      <x:c r="K72" s="26"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="26"/>
+      <x:c r="B73" s="26"/>
+      <x:c r="C73" s="26"/>
+      <x:c r="D73" s="26"/>
+      <x:c r="E73" s="26"/>
+      <x:c r="F73" s="26"/>
+      <x:c r="G73" s="26"/>
+      <x:c r="H73" s="26"/>
+      <x:c r="I73" s="26"/>
+      <x:c r="J73" s="26"/>
+      <x:c r="K73" s="26"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="26"/>
+      <x:c r="B74" s="26"/>
+      <x:c r="C74" s="26"/>
+      <x:c r="D74" s="26"/>
+      <x:c r="E74" s="26"/>
+      <x:c r="F74" s="26"/>
+      <x:c r="G74" s="26"/>
+      <x:c r="H74" s="26"/>
+      <x:c r="I74" s="26"/>
+      <x:c r="J74" s="26"/>
+      <x:c r="K74" s="26"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="26"/>
+      <x:c r="B75" s="26"/>
+      <x:c r="C75" s="26"/>
+      <x:c r="D75" s="26"/>
+      <x:c r="E75" s="26"/>
+      <x:c r="F75" s="26"/>
+      <x:c r="G75" s="26"/>
+      <x:c r="H75" s="26"/>
+      <x:c r="I75" s="26"/>
+      <x:c r="J75" s="26"/>
+      <x:c r="K75" s="26"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="26"/>
+      <x:c r="B76" s="26"/>
+      <x:c r="C76" s="26"/>
+      <x:c r="D76" s="26"/>
+      <x:c r="E76" s="26"/>
+      <x:c r="F76" s="26"/>
+      <x:c r="G76" s="26"/>
+      <x:c r="H76" s="26"/>
+      <x:c r="I76" s="26"/>
+      <x:c r="J76" s="26"/>
+      <x:c r="K76" s="26"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="26"/>
+      <x:c r="B77" s="26"/>
+      <x:c r="C77" s="26"/>
+      <x:c r="D77" s="26"/>
+      <x:c r="E77" s="26"/>
+      <x:c r="F77" s="26"/>
+      <x:c r="G77" s="26"/>
+      <x:c r="H77" s="26"/>
+      <x:c r="I77" s="26"/>
+      <x:c r="J77" s="26"/>
+      <x:c r="K77" s="26"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="26"/>
+      <x:c r="B78" s="26"/>
+      <x:c r="C78" s="26"/>
+      <x:c r="D78" s="26"/>
+      <x:c r="E78" s="26"/>
+      <x:c r="F78" s="26"/>
+      <x:c r="G78" s="26"/>
+      <x:c r="H78" s="26"/>
+      <x:c r="I78" s="26"/>
+      <x:c r="J78" s="26"/>
+      <x:c r="K78" s="26"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="26"/>
+      <x:c r="B79" s="26"/>
+      <x:c r="C79" s="26"/>
+      <x:c r="D79" s="26"/>
+      <x:c r="E79" s="26"/>
+      <x:c r="F79" s="26"/>
+      <x:c r="G79" s="26"/>
+      <x:c r="H79" s="26"/>
+      <x:c r="I79" s="26"/>
+      <x:c r="J79" s="26"/>
+      <x:c r="K79" s="26"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="26"/>
+      <x:c r="B80" s="26"/>
+      <x:c r="C80" s="26"/>
+      <x:c r="D80" s="26"/>
+      <x:c r="E80" s="26"/>
+      <x:c r="F80" s="26"/>
+      <x:c r="G80" s="26"/>
+      <x:c r="H80" s="26"/>
+      <x:c r="I80" s="26"/>
+      <x:c r="J80" s="26"/>
+      <x:c r="K80" s="26"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -1358,7 +2554,7 @@
         <x:v>schema_version</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>0.4</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>入力契約バージョン</x:v>

</xml_diff>

<commit_message>
archive slot-level homeroom boundary implementation
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,21 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rce4ae57acdfb44a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R0308edaba3fb495b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R7a74fc55705a42ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R5596ec139a5f40c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Re87ea8e2795b4752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R1ac5bae294f74ad5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R2efc711d8d0a4be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R73be8cafad4d4c48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R1a287a622e884461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R264f9bb3df35474e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R3d040cf4870b4dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R7ed81da29cae4872"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R3d27d55fe55c43b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="R333f07f4aa704b08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Rcd0b11a2534e4cd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rf0f21b6799d2451e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="Rb445c115c4f946ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rc7a0211c84ac4021"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="Rac9b0e8168c04f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R4f254ddccac543a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R15a7ccea68404c42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R5e4b098599c841ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R066f80d6b7f74583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="Rec939dd9393343b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="Raebb399b206c4bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R9a1f1f5b96a74f6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R9b8d1a4f5b5b4f49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R4f437d7e714b4fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Ra4541392f42f4bbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="R0cc73468c3a44ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_担任授業期間ルール" sheetId="16" r:id="R245828f3f3824d7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,7 +44,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -75,8 +76,18 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="6">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -106,11 +117,41 @@
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -164,6 +205,84 @@
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -1440,7 +1559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R282735b136654e9a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb44272aac05c445e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2529,6 +2648,70 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="27" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="38" t="str">
+        <x:v>rule_id</x:v>
+      </x:c>
+      <x:c r="B1" s="39" t="str">
+        <x:v>rule_name</x:v>
+      </x:c>
+      <x:c r="C1" s="39" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="D1" s="39" t="str">
+        <x:v>class_id</x:v>
+      </x:c>
+      <x:c r="E1" s="39" t="str">
+        <x:v>start_date</x:v>
+      </x:c>
+      <x:c r="F1" s="39" t="str">
+        <x:v>end_date</x:v>
+      </x:c>
+      <x:c r="G1" s="40" t="str">
+        <x:v>note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="47" t="str">
+        <x:v>HB_CL2_SAMPLE</x:v>
+      </x:c>
+      <x:c r="B2" s="48" t="str">
+        <x:v>サンプル期間の先頭・末尾を担任授業</x:v>
+      </x:c>
+      <x:c r="C2" s="51" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="48" t="str">
+        <x:v>CL2</x:v>
+      </x:c>
+      <x:c r="E2" s="52" t="n">
+        <x:v>46230</x:v>
+      </x:c>
+      <x:c r="F2" s="52" t="n">
+        <x:v>46231</x:v>
+      </x:c>
+      <x:c r="G2" s="50" t="str">
+        <x:v>H18のEnd-to-End確認用</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2554,7 +2737,7 @@
         <x:v>schema_version</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>0.6</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>入力契約バージョン</x:v>

</xml_diff>

<commit_message>
implement homeroom attendance boundaries; hold generation
実装・入力契約・独立検証・H18日単位境界ロジックと探索改善を保存。

現状: H18単体は成立するが、H11教師別校舎日制約との組合せで全42クラスの探索が長時間未確定。複数の局所修復・段階追加を試したが、実用的な生成時間で安定解に到達しないため、原因調査と実装をいったん保留する。

最終Excelは未生成。
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rf0f21b6799d2451e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="Rb445c115c4f946ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rc7a0211c84ac4021"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="Rac9b0e8168c04f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R4f254ddccac543a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R15a7ccea68404c42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R5e4b098599c841ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R066f80d6b7f74583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="Rec939dd9393343b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="Raebb399b206c4bcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R9a1f1f5b96a74f6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R9b8d1a4f5b5b4f49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R4f437d7e714b4fe4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Ra4541392f42f4bbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="R0cc73468c3a44ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_担任授業期間ルール" sheetId="16" r:id="R245828f3f3824d7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="R8e6ea8cdc6f340a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R16669c6c7f724767"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R6386904441c347d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R50d4ebc7150b46b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R3c9351f29aaa4204"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="Rd24095e2646945d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="Rf08001ab49bf4ad9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R1d8eb472f0b3440a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R3e3f58170d4a4c68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R5d40376e068a4771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R9d8894f59f274369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R049c634ddf9b4378"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R226858d1f6384a4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Rdf9a109cdfcb4abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Re93b57427a2e4727"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_担任授業期間ルール" sheetId="16" r:id="R510482e9b130458f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1559,7 +1559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb44272aac05c445e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe01b1be77244cfd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2689,7 +2689,7 @@
         <x:v>HB_CL2_SAMPLE</x:v>
       </x:c>
       <x:c r="B2" s="48" t="str">
-        <x:v>サンプル期間の先頭・末尾を担任授業</x:v>
+        <x:v>サンプル期間の初終登校日に担任授業</x:v>
       </x:c>
       <x:c r="C2" s="51" t="b">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Add flexible teacher day-off quotas
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,21 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rce4ae57acdfb44a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R0308edaba3fb495b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R7a74fc55705a42ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R5596ec139a5f40c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Re87ea8e2795b4752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R1ac5bae294f74ad5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R2efc711d8d0a4be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R73be8cafad4d4c48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R1a287a622e884461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R264f9bb3df35474e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R3d040cf4870b4dd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R7ed81da29cae4872"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R3d27d55fe55c43b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="R333f07f4aa704b08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Rcd0b11a2534e4cd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rf6f80fb442fe4684"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R8cd42e305af74b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R06535fe91281432e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R09e70b3120e747d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Rb5fabe0b58cf40ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="Rd89f02343ae244e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R9a0def33ddf14241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R3e65ba8a9f0b4d9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="Re8fca3a1640f465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R2213710f559e422d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R1b36288597234387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="Rcabc5aa53d91423e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Rf6ac78bd035f4a90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Reb15b78738aa493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Re4ef656923684fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="R8b892614f7394bd6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1440,7 +1441,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R282735b136654e9a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08d22fcd44004fa0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2529,6 +2530,47 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="6.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="7.78000020980835" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>rule_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>teacher_id</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>start_date</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>end_date</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>required_days_off</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>note</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>

</xml_diff>

<commit_message>
Add room priorities and input contract v0.7
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rf6f80fb442fe4684"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R8cd42e305af74b28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R06535fe91281432e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R09e70b3120e747d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Rb5fabe0b58cf40ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="Rd89f02343ae244e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R9a0def33ddf14241"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R3e65ba8a9f0b4d9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="Re8fca3a1640f465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R2213710f559e422d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R1b36288597234387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="Rcabc5aa53d91423e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Rf6ac78bd035f4a90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Reb15b78738aa493b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Re4ef656923684fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="R8b892614f7394bd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="R06a5c5a2f2794603"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="Rffcb1fc440a64db9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rca60f421a8f0468d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="Rc82726d16fe64eb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Rb1ef21a4261d4d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R2091396ec482409a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R5c443aa6151c478b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R4cd501a4548b4ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R701bf1857b324e11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R8b6a3cb6f2494ef3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R6342fece0d4940e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R27c440d4323746b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Rb6ce8d933bf846dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Rfd52b2296f574af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="R5eba9de7538045ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="R6dde0ea486d64a92"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -499,7 +499,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>時間割入力 v0.4</x:v>
+        <x:v>時間割入力 v0.7</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -520,6 +520,11 @@
     <x:row r="5">
       <x:c r="A5" t="str">
         <x:v>10_教師休みは、終日休みをALL、時限休みをP1|P2形式で入力します。行がない日時は勤務可能です。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>05_教室のpriorityは0以上の整数で、大きいほど優先します。同じ値の教室は横並びです。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1441,7 +1446,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08d22fcd44004fa0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49c2e5e84d0f41a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2596,7 +2601,7 @@
         <x:v>schema_version</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>0.6</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>入力契約バージョン</x:v>
@@ -3033,10 +3038,8 @@
           <x:t xml:space="preserve">C1</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第一校舎</x:t>
-        </x:is>
+      <x:c r="B2" t="str">
+        <x:v>六本松</x:v>
       </x:c>
       <x:c r="C2" t="n">
         <x:v>1</x:v>
@@ -3056,10 +3059,8 @@
           <x:t xml:space="preserve">C2</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第二校舎</x:t>
-        </x:is>
+      <x:c r="B3" t="str">
+        <x:v>梅光園</x:v>
       </x:c>
       <x:c r="C3" t="n">
         <x:v>2</x:v>
@@ -3082,129 +3083,125 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="6.440000057220459" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="9.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="8.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="9.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="6.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="3.7799999713897705" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">room_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">room_name</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">campus_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">output_order</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">enabled</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">note</x:t>
-        </x:is>
+      <x:c r="A1" t="str">
+        <x:v>room_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>room_name</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>campus_id</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>output_order</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>priority</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>note</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">101</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">C1</x:t>
-        </x:is>
+      <x:c r="A2" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="D2" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E2" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+      <x:c r="E2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>S19: なるべく空ける</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">102</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">C1</x:t>
-        </x:is>
+      <x:c r="A3" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>C1</x:v>
       </x:c>
       <x:c r="D3" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E3" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="E3" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F3" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G3"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">201</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">C2</x:t>
-        </x:is>
+      <x:c r="A4" t="str">
+        <x:v>R4</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="D4" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E4" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="E4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>S19: なるべく空ける</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>R3</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>C2</x:v>
+      </x:c>
+      <x:c r="D5" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F5" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add homeroom boundaries and flexible teacher day-off preferences
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,22 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="R06a5c5a2f2794603"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="Rffcb1fc440a64db9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="Rca60f421a8f0468d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="Rc82726d16fe64eb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Rb1ef21a4261d4d6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="R2091396ec482409a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R5c443aa6151c478b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R4cd501a4548b4ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R701bf1857b324e11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R8b6a3cb6f2494ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R6342fece0d4940e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R27c440d4323746b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Rb6ce8d933bf846dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="Rfd52b2296f574af7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="R5eba9de7538045ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="R6dde0ea486d64a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="R6feb44f4789445ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R657adca4a42e441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R404a7d7e7f40452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R240e389976594336"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Re76f1fca81884ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="Rb69f173b2c9a4af0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R60f6475f849444e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="Rdc75569583614886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="Re07e5d28115949c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R3da7fdf00a5e473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="Rc579639508c1433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="Ra50efe3350464ab0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Re2bd387fab5549ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="R3ec700c36c7e43df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Rab0ede4179db4736"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="Ra74a2ef853d94899"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_担任授業期間ルール" sheetId="17" r:id="R0ea6b42d2a01429a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31,7 +32,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -41,6 +42,11 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
@@ -111,7 +117,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -166,6 +172,16 @@
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1446,7 +1462,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49c2e5e84d0f41a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96e61c61b89348ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2539,13 +2555,18 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="7.78000020980835" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="7.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="32" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2568,10 +2589,1168 @@
         <x:v>required_days_off</x:v>
       </x:c>
       <x:c r="G1" t="str">
+        <x:v>minimum_days_off</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>maximum_days_off</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>preferred_days_off</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>quota_group_id</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>group_required_days_off</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
         <x:v>note</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="27" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="28" t="str">
+        <x:v>rule_id</x:v>
+      </x:c>
+      <x:c r="B1" s="28" t="str">
+        <x:v>rule_name</x:v>
+      </x:c>
+      <x:c r="C1" s="28" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="D1" s="28" t="str">
+        <x:v>condition_field</x:v>
+      </x:c>
+      <x:c r="E1" s="28" t="str">
+        <x:v>condition_operator</x:v>
+      </x:c>
+      <x:c r="F1" s="28" t="str">
+        <x:v>condition_value</x:v>
+      </x:c>
+      <x:c r="G1" s="28" t="str">
+        <x:v>start_date</x:v>
+      </x:c>
+      <x:c r="H1" s="28" t="str">
+        <x:v>end_date</x:v>
+      </x:c>
+      <x:c r="I1" s="28" t="str">
+        <x:v>note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="29"/>
+      <x:c r="B2" s="29"/>
+      <x:c r="C2" s="29"/>
+      <x:c r="D2" s="29"/>
+      <x:c r="E2" s="29"/>
+      <x:c r="F2" s="29"/>
+      <x:c r="G2" s="30"/>
+      <x:c r="H2" s="30"/>
+      <x:c r="I2" s="29"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="29"/>
+      <x:c r="B3" s="29"/>
+      <x:c r="C3" s="29"/>
+      <x:c r="D3" s="29"/>
+      <x:c r="E3" s="29"/>
+      <x:c r="F3" s="29"/>
+      <x:c r="G3" s="30"/>
+      <x:c r="H3" s="30"/>
+      <x:c r="I3" s="29"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="29"/>
+      <x:c r="B4" s="29"/>
+      <x:c r="C4" s="29"/>
+      <x:c r="D4" s="29"/>
+      <x:c r="E4" s="29"/>
+      <x:c r="F4" s="29"/>
+      <x:c r="G4" s="30"/>
+      <x:c r="H4" s="30"/>
+      <x:c r="I4" s="29"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="29"/>
+      <x:c r="B5" s="29"/>
+      <x:c r="C5" s="29"/>
+      <x:c r="D5" s="29"/>
+      <x:c r="E5" s="29"/>
+      <x:c r="F5" s="29"/>
+      <x:c r="G5" s="30"/>
+      <x:c r="H5" s="30"/>
+      <x:c r="I5" s="29"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="29"/>
+      <x:c r="B6" s="29"/>
+      <x:c r="C6" s="29"/>
+      <x:c r="D6" s="29"/>
+      <x:c r="E6" s="29"/>
+      <x:c r="F6" s="29"/>
+      <x:c r="G6" s="30"/>
+      <x:c r="H6" s="30"/>
+      <x:c r="I6" s="29"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="29"/>
+      <x:c r="B7" s="29"/>
+      <x:c r="C7" s="29"/>
+      <x:c r="D7" s="29"/>
+      <x:c r="E7" s="29"/>
+      <x:c r="F7" s="29"/>
+      <x:c r="G7" s="30"/>
+      <x:c r="H7" s="30"/>
+      <x:c r="I7" s="29"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="29"/>
+      <x:c r="B8" s="29"/>
+      <x:c r="C8" s="29"/>
+      <x:c r="D8" s="29"/>
+      <x:c r="E8" s="29"/>
+      <x:c r="F8" s="29"/>
+      <x:c r="G8" s="30"/>
+      <x:c r="H8" s="30"/>
+      <x:c r="I8" s="29"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="29"/>
+      <x:c r="B9" s="29"/>
+      <x:c r="C9" s="29"/>
+      <x:c r="D9" s="29"/>
+      <x:c r="E9" s="29"/>
+      <x:c r="F9" s="29"/>
+      <x:c r="G9" s="30"/>
+      <x:c r="H9" s="30"/>
+      <x:c r="I9" s="29"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="29"/>
+      <x:c r="B10" s="29"/>
+      <x:c r="C10" s="29"/>
+      <x:c r="D10" s="29"/>
+      <x:c r="E10" s="29"/>
+      <x:c r="F10" s="29"/>
+      <x:c r="G10" s="30"/>
+      <x:c r="H10" s="30"/>
+      <x:c r="I10" s="29"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="29"/>
+      <x:c r="B11" s="29"/>
+      <x:c r="C11" s="29"/>
+      <x:c r="D11" s="29"/>
+      <x:c r="E11" s="29"/>
+      <x:c r="F11" s="29"/>
+      <x:c r="G11" s="30"/>
+      <x:c r="H11" s="30"/>
+      <x:c r="I11" s="29"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="29"/>
+      <x:c r="B12" s="29"/>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29"/>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="29"/>
+      <x:c r="G12" s="30"/>
+      <x:c r="H12" s="30"/>
+      <x:c r="I12" s="29"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="29"/>
+      <x:c r="B13" s="29"/>
+      <x:c r="C13" s="29"/>
+      <x:c r="D13" s="29"/>
+      <x:c r="E13" s="29"/>
+      <x:c r="F13" s="29"/>
+      <x:c r="G13" s="30"/>
+      <x:c r="H13" s="30"/>
+      <x:c r="I13" s="29"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="29"/>
+      <x:c r="B14" s="29"/>
+      <x:c r="C14" s="29"/>
+      <x:c r="D14" s="29"/>
+      <x:c r="E14" s="29"/>
+      <x:c r="F14" s="29"/>
+      <x:c r="G14" s="30"/>
+      <x:c r="H14" s="30"/>
+      <x:c r="I14" s="29"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="29"/>
+      <x:c r="B15" s="29"/>
+      <x:c r="C15" s="29"/>
+      <x:c r="D15" s="29"/>
+      <x:c r="E15" s="29"/>
+      <x:c r="F15" s="29"/>
+      <x:c r="G15" s="30"/>
+      <x:c r="H15" s="30"/>
+      <x:c r="I15" s="29"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="29"/>
+      <x:c r="B16" s="29"/>
+      <x:c r="C16" s="29"/>
+      <x:c r="D16" s="29"/>
+      <x:c r="E16" s="29"/>
+      <x:c r="F16" s="29"/>
+      <x:c r="G16" s="30"/>
+      <x:c r="H16" s="30"/>
+      <x:c r="I16" s="29"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="29"/>
+      <x:c r="B17" s="29"/>
+      <x:c r="C17" s="29"/>
+      <x:c r="D17" s="29"/>
+      <x:c r="E17" s="29"/>
+      <x:c r="F17" s="29"/>
+      <x:c r="G17" s="30"/>
+      <x:c r="H17" s="30"/>
+      <x:c r="I17" s="29"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="29"/>
+      <x:c r="B18" s="29"/>
+      <x:c r="C18" s="29"/>
+      <x:c r="D18" s="29"/>
+      <x:c r="E18" s="29"/>
+      <x:c r="F18" s="29"/>
+      <x:c r="G18" s="30"/>
+      <x:c r="H18" s="30"/>
+      <x:c r="I18" s="29"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="29"/>
+      <x:c r="B19" s="29"/>
+      <x:c r="C19" s="29"/>
+      <x:c r="D19" s="29"/>
+      <x:c r="E19" s="29"/>
+      <x:c r="F19" s="29"/>
+      <x:c r="G19" s="30"/>
+      <x:c r="H19" s="30"/>
+      <x:c r="I19" s="29"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="29"/>
+      <x:c r="B20" s="29"/>
+      <x:c r="C20" s="29"/>
+      <x:c r="D20" s="29"/>
+      <x:c r="E20" s="29"/>
+      <x:c r="F20" s="29"/>
+      <x:c r="G20" s="30"/>
+      <x:c r="H20" s="30"/>
+      <x:c r="I20" s="29"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="29"/>
+      <x:c r="B21" s="29"/>
+      <x:c r="C21" s="29"/>
+      <x:c r="D21" s="29"/>
+      <x:c r="E21" s="29"/>
+      <x:c r="F21" s="29"/>
+      <x:c r="G21" s="30"/>
+      <x:c r="H21" s="30"/>
+      <x:c r="I21" s="29"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="29"/>
+      <x:c r="B22" s="29"/>
+      <x:c r="C22" s="29"/>
+      <x:c r="D22" s="29"/>
+      <x:c r="E22" s="29"/>
+      <x:c r="F22" s="29"/>
+      <x:c r="G22" s="30"/>
+      <x:c r="H22" s="30"/>
+      <x:c r="I22" s="29"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="29"/>
+      <x:c r="B23" s="29"/>
+      <x:c r="C23" s="29"/>
+      <x:c r="D23" s="29"/>
+      <x:c r="E23" s="29"/>
+      <x:c r="F23" s="29"/>
+      <x:c r="G23" s="30"/>
+      <x:c r="H23" s="30"/>
+      <x:c r="I23" s="29"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="29"/>
+      <x:c r="B24" s="29"/>
+      <x:c r="C24" s="29"/>
+      <x:c r="D24" s="29"/>
+      <x:c r="E24" s="29"/>
+      <x:c r="F24" s="29"/>
+      <x:c r="G24" s="30"/>
+      <x:c r="H24" s="30"/>
+      <x:c r="I24" s="29"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="29"/>
+      <x:c r="B25" s="29"/>
+      <x:c r="C25" s="29"/>
+      <x:c r="D25" s="29"/>
+      <x:c r="E25" s="29"/>
+      <x:c r="F25" s="29"/>
+      <x:c r="G25" s="30"/>
+      <x:c r="H25" s="30"/>
+      <x:c r="I25" s="29"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="29"/>
+      <x:c r="B26" s="29"/>
+      <x:c r="C26" s="29"/>
+      <x:c r="D26" s="29"/>
+      <x:c r="E26" s="29"/>
+      <x:c r="F26" s="29"/>
+      <x:c r="G26" s="30"/>
+      <x:c r="H26" s="30"/>
+      <x:c r="I26" s="29"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="29"/>
+      <x:c r="B27" s="29"/>
+      <x:c r="C27" s="29"/>
+      <x:c r="D27" s="29"/>
+      <x:c r="E27" s="29"/>
+      <x:c r="F27" s="29"/>
+      <x:c r="G27" s="30"/>
+      <x:c r="H27" s="30"/>
+      <x:c r="I27" s="29"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="29"/>
+      <x:c r="B28" s="29"/>
+      <x:c r="C28" s="29"/>
+      <x:c r="D28" s="29"/>
+      <x:c r="E28" s="29"/>
+      <x:c r="F28" s="29"/>
+      <x:c r="G28" s="30"/>
+      <x:c r="H28" s="30"/>
+      <x:c r="I28" s="29"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="29"/>
+      <x:c r="B29" s="29"/>
+      <x:c r="C29" s="29"/>
+      <x:c r="D29" s="29"/>
+      <x:c r="E29" s="29"/>
+      <x:c r="F29" s="29"/>
+      <x:c r="G29" s="30"/>
+      <x:c r="H29" s="30"/>
+      <x:c r="I29" s="29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="29"/>
+      <x:c r="B30" s="29"/>
+      <x:c r="C30" s="29"/>
+      <x:c r="D30" s="29"/>
+      <x:c r="E30" s="29"/>
+      <x:c r="F30" s="29"/>
+      <x:c r="G30" s="30"/>
+      <x:c r="H30" s="30"/>
+      <x:c r="I30" s="29"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="29"/>
+      <x:c r="B31" s="29"/>
+      <x:c r="C31" s="29"/>
+      <x:c r="D31" s="29"/>
+      <x:c r="E31" s="29"/>
+      <x:c r="F31" s="29"/>
+      <x:c r="G31" s="30"/>
+      <x:c r="H31" s="30"/>
+      <x:c r="I31" s="29"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="29"/>
+      <x:c r="B32" s="29"/>
+      <x:c r="C32" s="29"/>
+      <x:c r="D32" s="29"/>
+      <x:c r="E32" s="29"/>
+      <x:c r="F32" s="29"/>
+      <x:c r="G32" s="30"/>
+      <x:c r="H32" s="30"/>
+      <x:c r="I32" s="29"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="29"/>
+      <x:c r="B33" s="29"/>
+      <x:c r="C33" s="29"/>
+      <x:c r="D33" s="29"/>
+      <x:c r="E33" s="29"/>
+      <x:c r="F33" s="29"/>
+      <x:c r="G33" s="30"/>
+      <x:c r="H33" s="30"/>
+      <x:c r="I33" s="29"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="29"/>
+      <x:c r="B34" s="29"/>
+      <x:c r="C34" s="29"/>
+      <x:c r="D34" s="29"/>
+      <x:c r="E34" s="29"/>
+      <x:c r="F34" s="29"/>
+      <x:c r="G34" s="30"/>
+      <x:c r="H34" s="30"/>
+      <x:c r="I34" s="29"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="29"/>
+      <x:c r="B35" s="29"/>
+      <x:c r="C35" s="29"/>
+      <x:c r="D35" s="29"/>
+      <x:c r="E35" s="29"/>
+      <x:c r="F35" s="29"/>
+      <x:c r="G35" s="30"/>
+      <x:c r="H35" s="30"/>
+      <x:c r="I35" s="29"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="29"/>
+      <x:c r="B36" s="29"/>
+      <x:c r="C36" s="29"/>
+      <x:c r="D36" s="29"/>
+      <x:c r="E36" s="29"/>
+      <x:c r="F36" s="29"/>
+      <x:c r="G36" s="30"/>
+      <x:c r="H36" s="30"/>
+      <x:c r="I36" s="29"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="29"/>
+      <x:c r="B37" s="29"/>
+      <x:c r="C37" s="29"/>
+      <x:c r="D37" s="29"/>
+      <x:c r="E37" s="29"/>
+      <x:c r="F37" s="29"/>
+      <x:c r="G37" s="30"/>
+      <x:c r="H37" s="30"/>
+      <x:c r="I37" s="29"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="29"/>
+      <x:c r="B38" s="29"/>
+      <x:c r="C38" s="29"/>
+      <x:c r="D38" s="29"/>
+      <x:c r="E38" s="29"/>
+      <x:c r="F38" s="29"/>
+      <x:c r="G38" s="30"/>
+      <x:c r="H38" s="30"/>
+      <x:c r="I38" s="29"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="29"/>
+      <x:c r="B39" s="29"/>
+      <x:c r="C39" s="29"/>
+      <x:c r="D39" s="29"/>
+      <x:c r="E39" s="29"/>
+      <x:c r="F39" s="29"/>
+      <x:c r="G39" s="30"/>
+      <x:c r="H39" s="30"/>
+      <x:c r="I39" s="29"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="29"/>
+      <x:c r="B40" s="29"/>
+      <x:c r="C40" s="29"/>
+      <x:c r="D40" s="29"/>
+      <x:c r="E40" s="29"/>
+      <x:c r="F40" s="29"/>
+      <x:c r="G40" s="30"/>
+      <x:c r="H40" s="30"/>
+      <x:c r="I40" s="29"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="29"/>
+      <x:c r="B41" s="29"/>
+      <x:c r="C41" s="29"/>
+      <x:c r="D41" s="29"/>
+      <x:c r="E41" s="29"/>
+      <x:c r="F41" s="29"/>
+      <x:c r="G41" s="30"/>
+      <x:c r="H41" s="30"/>
+      <x:c r="I41" s="29"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="29"/>
+      <x:c r="B42" s="29"/>
+      <x:c r="C42" s="29"/>
+      <x:c r="D42" s="29"/>
+      <x:c r="E42" s="29"/>
+      <x:c r="F42" s="29"/>
+      <x:c r="G42" s="30"/>
+      <x:c r="H42" s="30"/>
+      <x:c r="I42" s="29"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="29"/>
+      <x:c r="B43" s="29"/>
+      <x:c r="C43" s="29"/>
+      <x:c r="D43" s="29"/>
+      <x:c r="E43" s="29"/>
+      <x:c r="F43" s="29"/>
+      <x:c r="G43" s="30"/>
+      <x:c r="H43" s="30"/>
+      <x:c r="I43" s="29"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="29"/>
+      <x:c r="B44" s="29"/>
+      <x:c r="C44" s="29"/>
+      <x:c r="D44" s="29"/>
+      <x:c r="E44" s="29"/>
+      <x:c r="F44" s="29"/>
+      <x:c r="G44" s="30"/>
+      <x:c r="H44" s="30"/>
+      <x:c r="I44" s="29"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="29"/>
+      <x:c r="B45" s="29"/>
+      <x:c r="C45" s="29"/>
+      <x:c r="D45" s="29"/>
+      <x:c r="E45" s="29"/>
+      <x:c r="F45" s="29"/>
+      <x:c r="G45" s="30"/>
+      <x:c r="H45" s="30"/>
+      <x:c r="I45" s="29"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="29"/>
+      <x:c r="B46" s="29"/>
+      <x:c r="C46" s="29"/>
+      <x:c r="D46" s="29"/>
+      <x:c r="E46" s="29"/>
+      <x:c r="F46" s="29"/>
+      <x:c r="G46" s="30"/>
+      <x:c r="H46" s="30"/>
+      <x:c r="I46" s="29"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="29"/>
+      <x:c r="B47" s="29"/>
+      <x:c r="C47" s="29"/>
+      <x:c r="D47" s="29"/>
+      <x:c r="E47" s="29"/>
+      <x:c r="F47" s="29"/>
+      <x:c r="G47" s="30"/>
+      <x:c r="H47" s="30"/>
+      <x:c r="I47" s="29"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="29"/>
+      <x:c r="B48" s="29"/>
+      <x:c r="C48" s="29"/>
+      <x:c r="D48" s="29"/>
+      <x:c r="E48" s="29"/>
+      <x:c r="F48" s="29"/>
+      <x:c r="G48" s="30"/>
+      <x:c r="H48" s="30"/>
+      <x:c r="I48" s="29"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="29"/>
+      <x:c r="B49" s="29"/>
+      <x:c r="C49" s="29"/>
+      <x:c r="D49" s="29"/>
+      <x:c r="E49" s="29"/>
+      <x:c r="F49" s="29"/>
+      <x:c r="G49" s="30"/>
+      <x:c r="H49" s="30"/>
+      <x:c r="I49" s="29"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="29"/>
+      <x:c r="B50" s="29"/>
+      <x:c r="C50" s="29"/>
+      <x:c r="D50" s="29"/>
+      <x:c r="E50" s="29"/>
+      <x:c r="F50" s="29"/>
+      <x:c r="G50" s="30"/>
+      <x:c r="H50" s="30"/>
+      <x:c r="I50" s="29"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="29"/>
+      <x:c r="B51" s="29"/>
+      <x:c r="C51" s="29"/>
+      <x:c r="D51" s="29"/>
+      <x:c r="E51" s="29"/>
+      <x:c r="F51" s="29"/>
+      <x:c r="G51" s="30"/>
+      <x:c r="H51" s="30"/>
+      <x:c r="I51" s="29"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="29"/>
+      <x:c r="B52" s="29"/>
+      <x:c r="C52" s="29"/>
+      <x:c r="D52" s="29"/>
+      <x:c r="E52" s="29"/>
+      <x:c r="F52" s="29"/>
+      <x:c r="G52" s="30"/>
+      <x:c r="H52" s="30"/>
+      <x:c r="I52" s="29"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="29"/>
+      <x:c r="B53" s="29"/>
+      <x:c r="C53" s="29"/>
+      <x:c r="D53" s="29"/>
+      <x:c r="E53" s="29"/>
+      <x:c r="F53" s="29"/>
+      <x:c r="G53" s="30"/>
+      <x:c r="H53" s="30"/>
+      <x:c r="I53" s="29"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="29"/>
+      <x:c r="B54" s="29"/>
+      <x:c r="C54" s="29"/>
+      <x:c r="D54" s="29"/>
+      <x:c r="E54" s="29"/>
+      <x:c r="F54" s="29"/>
+      <x:c r="G54" s="30"/>
+      <x:c r="H54" s="30"/>
+      <x:c r="I54" s="29"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="29"/>
+      <x:c r="B55" s="29"/>
+      <x:c r="C55" s="29"/>
+      <x:c r="D55" s="29"/>
+      <x:c r="E55" s="29"/>
+      <x:c r="F55" s="29"/>
+      <x:c r="G55" s="30"/>
+      <x:c r="H55" s="30"/>
+      <x:c r="I55" s="29"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="29"/>
+      <x:c r="B56" s="29"/>
+      <x:c r="C56" s="29"/>
+      <x:c r="D56" s="29"/>
+      <x:c r="E56" s="29"/>
+      <x:c r="F56" s="29"/>
+      <x:c r="G56" s="30"/>
+      <x:c r="H56" s="30"/>
+      <x:c r="I56" s="29"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="29"/>
+      <x:c r="B57" s="29"/>
+      <x:c r="C57" s="29"/>
+      <x:c r="D57" s="29"/>
+      <x:c r="E57" s="29"/>
+      <x:c r="F57" s="29"/>
+      <x:c r="G57" s="30"/>
+      <x:c r="H57" s="30"/>
+      <x:c r="I57" s="29"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="29"/>
+      <x:c r="B58" s="29"/>
+      <x:c r="C58" s="29"/>
+      <x:c r="D58" s="29"/>
+      <x:c r="E58" s="29"/>
+      <x:c r="F58" s="29"/>
+      <x:c r="G58" s="30"/>
+      <x:c r="H58" s="30"/>
+      <x:c r="I58" s="29"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="29"/>
+      <x:c r="B59" s="29"/>
+      <x:c r="C59" s="29"/>
+      <x:c r="D59" s="29"/>
+      <x:c r="E59" s="29"/>
+      <x:c r="F59" s="29"/>
+      <x:c r="G59" s="30"/>
+      <x:c r="H59" s="30"/>
+      <x:c r="I59" s="29"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="29"/>
+      <x:c r="B60" s="29"/>
+      <x:c r="C60" s="29"/>
+      <x:c r="D60" s="29"/>
+      <x:c r="E60" s="29"/>
+      <x:c r="F60" s="29"/>
+      <x:c r="G60" s="30"/>
+      <x:c r="H60" s="30"/>
+      <x:c r="I60" s="29"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="29"/>
+      <x:c r="B61" s="29"/>
+      <x:c r="C61" s="29"/>
+      <x:c r="D61" s="29"/>
+      <x:c r="E61" s="29"/>
+      <x:c r="F61" s="29"/>
+      <x:c r="G61" s="30"/>
+      <x:c r="H61" s="30"/>
+      <x:c r="I61" s="29"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="29"/>
+      <x:c r="B62" s="29"/>
+      <x:c r="C62" s="29"/>
+      <x:c r="D62" s="29"/>
+      <x:c r="E62" s="29"/>
+      <x:c r="F62" s="29"/>
+      <x:c r="G62" s="30"/>
+      <x:c r="H62" s="30"/>
+      <x:c r="I62" s="29"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="29"/>
+      <x:c r="B63" s="29"/>
+      <x:c r="C63" s="29"/>
+      <x:c r="D63" s="29"/>
+      <x:c r="E63" s="29"/>
+      <x:c r="F63" s="29"/>
+      <x:c r="G63" s="30"/>
+      <x:c r="H63" s="30"/>
+      <x:c r="I63" s="29"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="29"/>
+      <x:c r="B64" s="29"/>
+      <x:c r="C64" s="29"/>
+      <x:c r="D64" s="29"/>
+      <x:c r="E64" s="29"/>
+      <x:c r="F64" s="29"/>
+      <x:c r="G64" s="30"/>
+      <x:c r="H64" s="30"/>
+      <x:c r="I64" s="29"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="29"/>
+      <x:c r="B65" s="29"/>
+      <x:c r="C65" s="29"/>
+      <x:c r="D65" s="29"/>
+      <x:c r="E65" s="29"/>
+      <x:c r="F65" s="29"/>
+      <x:c r="G65" s="30"/>
+      <x:c r="H65" s="30"/>
+      <x:c r="I65" s="29"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="29"/>
+      <x:c r="B66" s="29"/>
+      <x:c r="C66" s="29"/>
+      <x:c r="D66" s="29"/>
+      <x:c r="E66" s="29"/>
+      <x:c r="F66" s="29"/>
+      <x:c r="G66" s="30"/>
+      <x:c r="H66" s="30"/>
+      <x:c r="I66" s="29"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="29"/>
+      <x:c r="B67" s="29"/>
+      <x:c r="C67" s="29"/>
+      <x:c r="D67" s="29"/>
+      <x:c r="E67" s="29"/>
+      <x:c r="F67" s="29"/>
+      <x:c r="G67" s="30"/>
+      <x:c r="H67" s="30"/>
+      <x:c r="I67" s="29"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="29"/>
+      <x:c r="B68" s="29"/>
+      <x:c r="C68" s="29"/>
+      <x:c r="D68" s="29"/>
+      <x:c r="E68" s="29"/>
+      <x:c r="F68" s="29"/>
+      <x:c r="G68" s="30"/>
+      <x:c r="H68" s="30"/>
+      <x:c r="I68" s="29"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="29"/>
+      <x:c r="B69" s="29"/>
+      <x:c r="C69" s="29"/>
+      <x:c r="D69" s="29"/>
+      <x:c r="E69" s="29"/>
+      <x:c r="F69" s="29"/>
+      <x:c r="G69" s="30"/>
+      <x:c r="H69" s="30"/>
+      <x:c r="I69" s="29"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="29"/>
+      <x:c r="B70" s="29"/>
+      <x:c r="C70" s="29"/>
+      <x:c r="D70" s="29"/>
+      <x:c r="E70" s="29"/>
+      <x:c r="F70" s="29"/>
+      <x:c r="G70" s="30"/>
+      <x:c r="H70" s="30"/>
+      <x:c r="I70" s="29"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="29"/>
+      <x:c r="B71" s="29"/>
+      <x:c r="C71" s="29"/>
+      <x:c r="D71" s="29"/>
+      <x:c r="E71" s="29"/>
+      <x:c r="F71" s="29"/>
+      <x:c r="G71" s="30"/>
+      <x:c r="H71" s="30"/>
+      <x:c r="I71" s="29"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="29"/>
+      <x:c r="B72" s="29"/>
+      <x:c r="C72" s="29"/>
+      <x:c r="D72" s="29"/>
+      <x:c r="E72" s="29"/>
+      <x:c r="F72" s="29"/>
+      <x:c r="G72" s="30"/>
+      <x:c r="H72" s="30"/>
+      <x:c r="I72" s="29"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="29"/>
+      <x:c r="B73" s="29"/>
+      <x:c r="C73" s="29"/>
+      <x:c r="D73" s="29"/>
+      <x:c r="E73" s="29"/>
+      <x:c r="F73" s="29"/>
+      <x:c r="G73" s="30"/>
+      <x:c r="H73" s="30"/>
+      <x:c r="I73" s="29"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="29"/>
+      <x:c r="B74" s="29"/>
+      <x:c r="C74" s="29"/>
+      <x:c r="D74" s="29"/>
+      <x:c r="E74" s="29"/>
+      <x:c r="F74" s="29"/>
+      <x:c r="G74" s="30"/>
+      <x:c r="H74" s="30"/>
+      <x:c r="I74" s="29"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="29"/>
+      <x:c r="B75" s="29"/>
+      <x:c r="C75" s="29"/>
+      <x:c r="D75" s="29"/>
+      <x:c r="E75" s="29"/>
+      <x:c r="F75" s="29"/>
+      <x:c r="G75" s="30"/>
+      <x:c r="H75" s="30"/>
+      <x:c r="I75" s="29"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="29"/>
+      <x:c r="B76" s="29"/>
+      <x:c r="C76" s="29"/>
+      <x:c r="D76" s="29"/>
+      <x:c r="E76" s="29"/>
+      <x:c r="F76" s="29"/>
+      <x:c r="G76" s="30"/>
+      <x:c r="H76" s="30"/>
+      <x:c r="I76" s="29"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="29"/>
+      <x:c r="B77" s="29"/>
+      <x:c r="C77" s="29"/>
+      <x:c r="D77" s="29"/>
+      <x:c r="E77" s="29"/>
+      <x:c r="F77" s="29"/>
+      <x:c r="G77" s="30"/>
+      <x:c r="H77" s="30"/>
+      <x:c r="I77" s="29"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="29"/>
+      <x:c r="B78" s="29"/>
+      <x:c r="C78" s="29"/>
+      <x:c r="D78" s="29"/>
+      <x:c r="E78" s="29"/>
+      <x:c r="F78" s="29"/>
+      <x:c r="G78" s="30"/>
+      <x:c r="H78" s="30"/>
+      <x:c r="I78" s="29"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="29"/>
+      <x:c r="B79" s="29"/>
+      <x:c r="C79" s="29"/>
+      <x:c r="D79" s="29"/>
+      <x:c r="E79" s="29"/>
+      <x:c r="F79" s="29"/>
+      <x:c r="G79" s="30"/>
+      <x:c r="H79" s="30"/>
+      <x:c r="I79" s="29"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="29"/>
+      <x:c r="B80" s="29"/>
+      <x:c r="C80" s="29"/>
+      <x:c r="D80" s="29"/>
+      <x:c r="E80" s="29"/>
+      <x:c r="F80" s="29"/>
+      <x:c r="G80" s="30"/>
+      <x:c r="H80" s="30"/>
+      <x:c r="I80" s="29"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="29"/>
+      <x:c r="B81" s="29"/>
+      <x:c r="C81" s="29"/>
+      <x:c r="D81" s="29"/>
+      <x:c r="E81" s="29"/>
+      <x:c r="F81" s="29"/>
+      <x:c r="G81" s="30"/>
+      <x:c r="H81" s="30"/>
+      <x:c r="I81" s="29"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="29"/>
+      <x:c r="B82" s="29"/>
+      <x:c r="C82" s="29"/>
+      <x:c r="D82" s="29"/>
+      <x:c r="E82" s="29"/>
+      <x:c r="F82" s="29"/>
+      <x:c r="G82" s="30"/>
+      <x:c r="H82" s="30"/>
+      <x:c r="I82" s="29"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="29"/>
+      <x:c r="B83" s="29"/>
+      <x:c r="C83" s="29"/>
+      <x:c r="D83" s="29"/>
+      <x:c r="E83" s="29"/>
+      <x:c r="F83" s="29"/>
+      <x:c r="G83" s="30"/>
+      <x:c r="H83" s="30"/>
+      <x:c r="I83" s="29"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="29"/>
+      <x:c r="B84" s="29"/>
+      <x:c r="C84" s="29"/>
+      <x:c r="D84" s="29"/>
+      <x:c r="E84" s="29"/>
+      <x:c r="F84" s="29"/>
+      <x:c r="G84" s="30"/>
+      <x:c r="H84" s="30"/>
+      <x:c r="I84" s="29"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="29"/>
+      <x:c r="B85" s="29"/>
+      <x:c r="C85" s="29"/>
+      <x:c r="D85" s="29"/>
+      <x:c r="E85" s="29"/>
+      <x:c r="F85" s="29"/>
+      <x:c r="G85" s="30"/>
+      <x:c r="H85" s="30"/>
+      <x:c r="I85" s="29"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="29"/>
+      <x:c r="B86" s="29"/>
+      <x:c r="C86" s="29"/>
+      <x:c r="D86" s="29"/>
+      <x:c r="E86" s="29"/>
+      <x:c r="F86" s="29"/>
+      <x:c r="G86" s="30"/>
+      <x:c r="H86" s="30"/>
+      <x:c r="I86" s="29"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="29"/>
+      <x:c r="B87" s="29"/>
+      <x:c r="C87" s="29"/>
+      <x:c r="D87" s="29"/>
+      <x:c r="E87" s="29"/>
+      <x:c r="F87" s="29"/>
+      <x:c r="G87" s="30"/>
+      <x:c r="H87" s="30"/>
+      <x:c r="I87" s="29"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="29"/>
+      <x:c r="B88" s="29"/>
+      <x:c r="C88" s="29"/>
+      <x:c r="D88" s="29"/>
+      <x:c r="E88" s="29"/>
+      <x:c r="F88" s="29"/>
+      <x:c r="G88" s="30"/>
+      <x:c r="H88" s="30"/>
+      <x:c r="I88" s="29"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="29"/>
+      <x:c r="B89" s="29"/>
+      <x:c r="C89" s="29"/>
+      <x:c r="D89" s="29"/>
+      <x:c r="E89" s="29"/>
+      <x:c r="F89" s="29"/>
+      <x:c r="G89" s="30"/>
+      <x:c r="H89" s="30"/>
+      <x:c r="I89" s="29"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="29"/>
+      <x:c r="B90" s="29"/>
+      <x:c r="C90" s="29"/>
+      <x:c r="D90" s="29"/>
+      <x:c r="E90" s="29"/>
+      <x:c r="F90" s="29"/>
+      <x:c r="G90" s="30"/>
+      <x:c r="H90" s="30"/>
+      <x:c r="I90" s="29"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="29"/>
+      <x:c r="B91" s="29"/>
+      <x:c r="C91" s="29"/>
+      <x:c r="D91" s="29"/>
+      <x:c r="E91" s="29"/>
+      <x:c r="F91" s="29"/>
+      <x:c r="G91" s="30"/>
+      <x:c r="H91" s="30"/>
+      <x:c r="I91" s="29"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="29"/>
+      <x:c r="B92" s="29"/>
+      <x:c r="C92" s="29"/>
+      <x:c r="D92" s="29"/>
+      <x:c r="E92" s="29"/>
+      <x:c r="F92" s="29"/>
+      <x:c r="G92" s="30"/>
+      <x:c r="H92" s="30"/>
+      <x:c r="I92" s="29"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="29"/>
+      <x:c r="B93" s="29"/>
+      <x:c r="C93" s="29"/>
+      <x:c r="D93" s="29"/>
+      <x:c r="E93" s="29"/>
+      <x:c r="F93" s="29"/>
+      <x:c r="G93" s="30"/>
+      <x:c r="H93" s="30"/>
+      <x:c r="I93" s="29"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="29"/>
+      <x:c r="B94" s="29"/>
+      <x:c r="C94" s="29"/>
+      <x:c r="D94" s="29"/>
+      <x:c r="E94" s="29"/>
+      <x:c r="F94" s="29"/>
+      <x:c r="G94" s="30"/>
+      <x:c r="H94" s="30"/>
+      <x:c r="I94" s="29"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="29"/>
+      <x:c r="B95" s="29"/>
+      <x:c r="C95" s="29"/>
+      <x:c r="D95" s="29"/>
+      <x:c r="E95" s="29"/>
+      <x:c r="F95" s="29"/>
+      <x:c r="G95" s="30"/>
+      <x:c r="H95" s="30"/>
+      <x:c r="I95" s="29"/>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="29"/>
+      <x:c r="B96" s="29"/>
+      <x:c r="C96" s="29"/>
+      <x:c r="D96" s="29"/>
+      <x:c r="E96" s="29"/>
+      <x:c r="F96" s="29"/>
+      <x:c r="G96" s="30"/>
+      <x:c r="H96" s="30"/>
+      <x:c r="I96" s="29"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="29"/>
+      <x:c r="B97" s="29"/>
+      <x:c r="C97" s="29"/>
+      <x:c r="D97" s="29"/>
+      <x:c r="E97" s="29"/>
+      <x:c r="F97" s="29"/>
+      <x:c r="G97" s="30"/>
+      <x:c r="H97" s="30"/>
+      <x:c r="I97" s="29"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="29"/>
+      <x:c r="B98" s="29"/>
+      <x:c r="C98" s="29"/>
+      <x:c r="D98" s="29"/>
+      <x:c r="E98" s="29"/>
+      <x:c r="F98" s="29"/>
+      <x:c r="G98" s="30"/>
+      <x:c r="H98" s="30"/>
+      <x:c r="I98" s="29"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="29"/>
+      <x:c r="B99" s="29"/>
+      <x:c r="C99" s="29"/>
+      <x:c r="D99" s="29"/>
+      <x:c r="E99" s="29"/>
+      <x:c r="F99" s="29"/>
+      <x:c r="G99" s="30"/>
+      <x:c r="H99" s="30"/>
+      <x:c r="I99" s="29"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="29"/>
+      <x:c r="B100" s="29"/>
+      <x:c r="C100" s="29"/>
+      <x:c r="D100" s="29"/>
+      <x:c r="E100" s="29"/>
+      <x:c r="F100" s="29"/>
+      <x:c r="G100" s="30"/>
+      <x:c r="H100" s="30"/>
+      <x:c r="I100" s="29"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C2:C100">
+      <x:formula1>"true,false"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -2601,7 +3780,7 @@
         <x:v>schema_version</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>0.7</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>入力契約バージョン</x:v>
@@ -3445,12 +4624,15 @@
           <x:t xml:space="preserve">subject_name</x:t>
         </x:is>
       </x:c>
-      <x:c r="C1" t="inlineStr">
+      <x:c r="C1" t="str">
+        <x:v>lesson_type</x:v>
+      </x:c>
+      <x:c r="D1" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">enabled</x:t>
         </x:is>
       </x:c>
-      <x:c r="D1" t="inlineStr">
+      <x:c r="E1" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">note</x:t>
         </x:is>
@@ -3467,14 +4649,13 @@
           <x:t xml:space="preserve">算数</x:t>
         </x:is>
       </x:c>
-      <x:c r="C2" t="b">
+      <x:c r="C2" t="str">
+        <x:v>regular</x:v>
+      </x:c>
+      <x:c r="D2" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="E2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="inlineStr">
@@ -3487,16 +4668,20 @@
           <x:t xml:space="preserve">英語</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" t="b">
+      <x:c r="C3" t="str">
+        <x:v>regular</x:v>
+      </x:c>
+      <x:c r="D3" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="E3"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C2:C200">
+      <x:formula1>"regular,special,other"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add required class lesson slots and refine teacher span rule
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="R6feb44f4789445ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R657adca4a42e441e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R404a7d7e7f40452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R240e389976594336"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="Re76f1fca81884ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="Rb69f173b2c9a4af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R60f6475f849444e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="Rdc75569583614886"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="Re07e5d28115949c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R3da7fdf00a5e473f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="Rc579639508c1433f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="Ra50efe3350464ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Re2bd387fab5549ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="R3ec700c36c7e43df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Rab0ede4179db4736"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="Ra74a2ef853d94899"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_担任授業期間ルール" sheetId="17" r:id="R0ea6b42d2a01429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Re05f306aec3e463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="Rc403fd97942b45c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R5a91f56d5cb84a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R8d73821883934440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R22f3b8dabb044c9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="Rfcc00a6be2dd416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R73c5ecd6c8a045f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R28297a060f8343e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R7d008b78fa2d46d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R1f5e7957ebf5412a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R614cff841ad246a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R61079fcad7844d41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R94ab07ed12664ce5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="R81275d3652fe4f02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="R1326e5bd1a004d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="R976f9884f35d4771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_担任授業期間ルール" sheetId="17" r:id="R96a728fc8ac1489d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -831,312 +831,178 @@
     <x:col min="17" max="17" width="5.559999942779541" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="3.7799999713897705" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="31" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">rule_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">rule_name</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">enabled</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">constraint_type</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">target_entity</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">condition_field</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">condition_operator</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">condition_value</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">campus_id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">start_date</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">end_date</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">weekdays</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">allowed_periods</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">daily_hard_limit</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">consecutive_limit</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">attendance_streak_limit</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">priority</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">note</x:t>
-        </x:is>
+      <x:c r="A1" t="str">
+        <x:v>rule_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>rule_name</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>constraint_type</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>target_entity</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>condition_field</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>condition_operator</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>condition_value</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>campus_id</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>start_date</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>end_date</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>weekdays</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>allowed_periods</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>daily_hard_limit</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>forbid_first_last_same_day</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>attendance_streak_limit</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>priority</x:v>
+      </x:c>
+      <x:c r="R1" t="str">
+        <x:v>note</x:v>
       </x:c>
       <x:c r="S1" t="str">
         <x:v>preferred_attendance_streak_limit</x:v>
       </x:c>
+      <x:c r="T1" t="str">
+        <x:v>required_lesson_periods</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R_CLASS_BASE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">クラス共通</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" t="b">
+      <x:c r="A2" t="str">
+        <x:v>R_CLASS_BASE</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>クラス共通</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">hard</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">class</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="I2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="J2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="K2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="L2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="M2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1|P2|P3|P4|P5|P6</x:t>
-        </x:is>
+      <x:c r="D2" t="str">
+        <x:v>hard</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>class</x:v>
+      </x:c>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2" t="str">
+        <x:v>P1|P2|P3|P4|P5|P6</x:v>
       </x:c>
       <x:c r="N2" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="O2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="O2"/>
       <x:c r="P2"/>
       <x:c r="Q2" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="R2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="R2"/>
+      <x:c r="S2"/>
+      <x:c r="T2"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R_ELEMENTARY</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">小学部許可時限</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" t="b">
+      <x:c r="A3" t="str">
+        <x:v>R_ELEMENTARY</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>小学部許可時限</x:v>
+      </x:c>
+      <x:c r="C3" s="8" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">hard</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">class</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">division</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">eq</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">elementary</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="J3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="K3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="L3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="M3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P1|P2|P3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="O3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>hard</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>class</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>division</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>eq</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>elementary</x:v>
+      </x:c>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
+      <x:c r="M3" t="str">
+        <x:v>P1|P2|P3</x:v>
+      </x:c>
+      <x:c r="N3"/>
+      <x:c r="O3"/>
       <x:c r="P3"/>
       <x:c r="Q3" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="R3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="R3"/>
+      <x:c r="S3"/>
+      <x:c r="T3"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R_JH_OVERRIDE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中学部指定日override</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" t="b">
+      <x:c r="A4" t="str">
+        <x:v>R_JH_OVERRIDE</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>中学部指定日override</x:v>
+      </x:c>
+      <x:c r="C4" s="8" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">override</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">class</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">division|grade</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">eq|between</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">junior_high|1/3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">C2</x:t>
-        </x:is>
+      <x:c r="D4" t="str">
+        <x:v>override</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>class</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>division|grade</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>eq|between</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>junior_high|1/3</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>C2</x:v>
       </x:c>
       <x:c r="J4" s="1" t="n">
         <x:v>46231</x:v>
@@ -1144,117 +1010,61 @@
       <x:c r="K4" s="1" t="n">
         <x:v>46231</x:v>
       </x:c>
-      <x:c r="L4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TUE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P4|P5|P6</x:t>
-        </x:is>
+      <x:c r="L4" t="str">
+        <x:v>TUE</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>P4|P5|P6</x:v>
       </x:c>
       <x:c r="N4" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="O4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="O4"/>
       <x:c r="P4"/>
       <x:c r="Q4" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="R4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="R4"/>
+      <x:c r="S4"/>
+      <x:c r="T4"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R_TEACHER_BASE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">教師共通</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" t="b">
+      <x:c r="A5" t="str">
+        <x:v>R_TEACHER_BASE</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>教師共通</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">hard</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">teacher</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="G5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="H5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="I5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="J5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="K5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="L5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="M5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>hard</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>teacher</x:v>
+      </x:c>
+      <x:c r="F5"/>
+      <x:c r="G5"/>
+      <x:c r="H5"/>
+      <x:c r="I5"/>
+      <x:c r="J5"/>
+      <x:c r="K5"/>
+      <x:c r="L5"/>
+      <x:c r="M5"/>
       <x:c r="N5" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="O5" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="O5" s="8" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P5"/>
       <x:c r="Q5" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="R5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="R5"/>
+      <x:c r="S5"/>
+      <x:c r="T5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
@@ -1298,6 +1108,7 @@
       <x:c r="S6" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="T6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
@@ -1343,6 +1154,2986 @@
       <x:c r="S7" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="T7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="T8"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="T9"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="T10"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="T11"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="T12"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="T13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="T14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="T15"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="T16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="T17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="T18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="T19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="T20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="T21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="T22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="T23"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="T24"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="T25"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="T26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="T27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="T28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="T29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="T30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="T31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="T32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="T33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="T34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="T35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="T36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="T37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="T38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="T39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="T40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="T41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="T42"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="T43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="T44"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="T45"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="T46"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="T47"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="T48"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="T49"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="T50"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="T51"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="T52"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="T53"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="T54"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="T55"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="T56"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="T57"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="T58"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="T59"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="T60"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="T61"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="T62"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="T63"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="T64"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="T65"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="T66"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="T67"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="T68"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="T69"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="T70"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="T71"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="T72"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="T73"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="T74"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="T75"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="T76"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="T77"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="T78"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="T79"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="T80"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="T81"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="T82"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="T83"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="T84"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="T85"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="T86"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="T87"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="T88"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="T89"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="T90"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="T91"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="T92"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="T93"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="T94"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="T95"/>
+    </x:row>
+    <x:row r="96">
+      <x:c r="T96"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="T97"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="T98"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="T99"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="T100"/>
+    </x:row>
+    <x:row r="101">
+      <x:c r="T101"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="T102"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="T103"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="T104"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="T105"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="T106"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="T107"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="T108"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="T109"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="T110"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="T111"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="T112"/>
+    </x:row>
+    <x:row r="113">
+      <x:c r="T113"/>
+    </x:row>
+    <x:row r="114">
+      <x:c r="T114"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="T115"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="T116"/>
+    </x:row>
+    <x:row r="117">
+      <x:c r="T117"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="T118"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="T119"/>
+    </x:row>
+    <x:row r="120">
+      <x:c r="T120"/>
+    </x:row>
+    <x:row r="121">
+      <x:c r="T121"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="T122"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="T123"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="T124"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="T125"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="T126"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="T127"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="T128"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="T129"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="T130"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="T131"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="T132"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="T133"/>
+    </x:row>
+    <x:row r="134">
+      <x:c r="T134"/>
+    </x:row>
+    <x:row r="135">
+      <x:c r="T135"/>
+    </x:row>
+    <x:row r="136">
+      <x:c r="T136"/>
+    </x:row>
+    <x:row r="137">
+      <x:c r="T137"/>
+    </x:row>
+    <x:row r="138">
+      <x:c r="T138"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="T139"/>
+    </x:row>
+    <x:row r="140">
+      <x:c r="T140"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="T141"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="T142"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="T143"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="T144"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="T145"/>
+    </x:row>
+    <x:row r="146">
+      <x:c r="T146"/>
+    </x:row>
+    <x:row r="147">
+      <x:c r="T147"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="T148"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="T149"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="T150"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="T151"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="T152"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="T153"/>
+    </x:row>
+    <x:row r="154">
+      <x:c r="T154"/>
+    </x:row>
+    <x:row r="155">
+      <x:c r="T155"/>
+    </x:row>
+    <x:row r="156">
+      <x:c r="T156"/>
+    </x:row>
+    <x:row r="157">
+      <x:c r="T157"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="T158"/>
+    </x:row>
+    <x:row r="159">
+      <x:c r="T159"/>
+    </x:row>
+    <x:row r="160">
+      <x:c r="T160"/>
+    </x:row>
+    <x:row r="161">
+      <x:c r="T161"/>
+    </x:row>
+    <x:row r="162">
+      <x:c r="T162"/>
+    </x:row>
+    <x:row r="163">
+      <x:c r="T163"/>
+    </x:row>
+    <x:row r="164">
+      <x:c r="T164"/>
+    </x:row>
+    <x:row r="165">
+      <x:c r="T165"/>
+    </x:row>
+    <x:row r="166">
+      <x:c r="T166"/>
+    </x:row>
+    <x:row r="167">
+      <x:c r="T167"/>
+    </x:row>
+    <x:row r="168">
+      <x:c r="T168"/>
+    </x:row>
+    <x:row r="169">
+      <x:c r="T169"/>
+    </x:row>
+    <x:row r="170">
+      <x:c r="T170"/>
+    </x:row>
+    <x:row r="171">
+      <x:c r="T171"/>
+    </x:row>
+    <x:row r="172">
+      <x:c r="T172"/>
+    </x:row>
+    <x:row r="173">
+      <x:c r="T173"/>
+    </x:row>
+    <x:row r="174">
+      <x:c r="T174"/>
+    </x:row>
+    <x:row r="175">
+      <x:c r="T175"/>
+    </x:row>
+    <x:row r="176">
+      <x:c r="T176"/>
+    </x:row>
+    <x:row r="177">
+      <x:c r="T177"/>
+    </x:row>
+    <x:row r="178">
+      <x:c r="T178"/>
+    </x:row>
+    <x:row r="179">
+      <x:c r="T179"/>
+    </x:row>
+    <x:row r="180">
+      <x:c r="T180"/>
+    </x:row>
+    <x:row r="181">
+      <x:c r="T181"/>
+    </x:row>
+    <x:row r="182">
+      <x:c r="T182"/>
+    </x:row>
+    <x:row r="183">
+      <x:c r="T183"/>
+    </x:row>
+    <x:row r="184">
+      <x:c r="T184"/>
+    </x:row>
+    <x:row r="185">
+      <x:c r="T185"/>
+    </x:row>
+    <x:row r="186">
+      <x:c r="T186"/>
+    </x:row>
+    <x:row r="187">
+      <x:c r="T187"/>
+    </x:row>
+    <x:row r="188">
+      <x:c r="T188"/>
+    </x:row>
+    <x:row r="189">
+      <x:c r="T189"/>
+    </x:row>
+    <x:row r="190">
+      <x:c r="T190"/>
+    </x:row>
+    <x:row r="191">
+      <x:c r="T191"/>
+    </x:row>
+    <x:row r="192">
+      <x:c r="T192"/>
+    </x:row>
+    <x:row r="193">
+      <x:c r="T193"/>
+    </x:row>
+    <x:row r="194">
+      <x:c r="T194"/>
+    </x:row>
+    <x:row r="195">
+      <x:c r="T195"/>
+    </x:row>
+    <x:row r="196">
+      <x:c r="T196"/>
+    </x:row>
+    <x:row r="197">
+      <x:c r="T197"/>
+    </x:row>
+    <x:row r="198">
+      <x:c r="T198"/>
+    </x:row>
+    <x:row r="199">
+      <x:c r="T199"/>
+    </x:row>
+    <x:row r="200">
+      <x:c r="T200"/>
+    </x:row>
+    <x:row r="201">
+      <x:c r="T201"/>
+    </x:row>
+    <x:row r="202">
+      <x:c r="T202"/>
+    </x:row>
+    <x:row r="203">
+      <x:c r="T203"/>
+    </x:row>
+    <x:row r="204">
+      <x:c r="T204"/>
+    </x:row>
+    <x:row r="205">
+      <x:c r="T205"/>
+    </x:row>
+    <x:row r="206">
+      <x:c r="T206"/>
+    </x:row>
+    <x:row r="207">
+      <x:c r="T207"/>
+    </x:row>
+    <x:row r="208">
+      <x:c r="T208"/>
+    </x:row>
+    <x:row r="209">
+      <x:c r="T209"/>
+    </x:row>
+    <x:row r="210">
+      <x:c r="T210"/>
+    </x:row>
+    <x:row r="211">
+      <x:c r="T211"/>
+    </x:row>
+    <x:row r="212">
+      <x:c r="T212"/>
+    </x:row>
+    <x:row r="213">
+      <x:c r="T213"/>
+    </x:row>
+    <x:row r="214">
+      <x:c r="T214"/>
+    </x:row>
+    <x:row r="215">
+      <x:c r="T215"/>
+    </x:row>
+    <x:row r="216">
+      <x:c r="T216"/>
+    </x:row>
+    <x:row r="217">
+      <x:c r="T217"/>
+    </x:row>
+    <x:row r="218">
+      <x:c r="T218"/>
+    </x:row>
+    <x:row r="219">
+      <x:c r="T219"/>
+    </x:row>
+    <x:row r="220">
+      <x:c r="T220"/>
+    </x:row>
+    <x:row r="221">
+      <x:c r="T221"/>
+    </x:row>
+    <x:row r="222">
+      <x:c r="T222"/>
+    </x:row>
+    <x:row r="223">
+      <x:c r="T223"/>
+    </x:row>
+    <x:row r="224">
+      <x:c r="T224"/>
+    </x:row>
+    <x:row r="225">
+      <x:c r="T225"/>
+    </x:row>
+    <x:row r="226">
+      <x:c r="T226"/>
+    </x:row>
+    <x:row r="227">
+      <x:c r="T227"/>
+    </x:row>
+    <x:row r="228">
+      <x:c r="T228"/>
+    </x:row>
+    <x:row r="229">
+      <x:c r="T229"/>
+    </x:row>
+    <x:row r="230">
+      <x:c r="T230"/>
+    </x:row>
+    <x:row r="231">
+      <x:c r="T231"/>
+    </x:row>
+    <x:row r="232">
+      <x:c r="T232"/>
+    </x:row>
+    <x:row r="233">
+      <x:c r="T233"/>
+    </x:row>
+    <x:row r="234">
+      <x:c r="T234"/>
+    </x:row>
+    <x:row r="235">
+      <x:c r="T235"/>
+    </x:row>
+    <x:row r="236">
+      <x:c r="T236"/>
+    </x:row>
+    <x:row r="237">
+      <x:c r="T237"/>
+    </x:row>
+    <x:row r="238">
+      <x:c r="T238"/>
+    </x:row>
+    <x:row r="239">
+      <x:c r="T239"/>
+    </x:row>
+    <x:row r="240">
+      <x:c r="T240"/>
+    </x:row>
+    <x:row r="241">
+      <x:c r="T241"/>
+    </x:row>
+    <x:row r="242">
+      <x:c r="T242"/>
+    </x:row>
+    <x:row r="243">
+      <x:c r="T243"/>
+    </x:row>
+    <x:row r="244">
+      <x:c r="T244"/>
+    </x:row>
+    <x:row r="245">
+      <x:c r="T245"/>
+    </x:row>
+    <x:row r="246">
+      <x:c r="T246"/>
+    </x:row>
+    <x:row r="247">
+      <x:c r="T247"/>
+    </x:row>
+    <x:row r="248">
+      <x:c r="T248"/>
+    </x:row>
+    <x:row r="249">
+      <x:c r="T249"/>
+    </x:row>
+    <x:row r="250">
+      <x:c r="T250"/>
+    </x:row>
+    <x:row r="251">
+      <x:c r="T251"/>
+    </x:row>
+    <x:row r="252">
+      <x:c r="T252"/>
+    </x:row>
+    <x:row r="253">
+      <x:c r="T253"/>
+    </x:row>
+    <x:row r="254">
+      <x:c r="T254"/>
+    </x:row>
+    <x:row r="255">
+      <x:c r="T255"/>
+    </x:row>
+    <x:row r="256">
+      <x:c r="T256"/>
+    </x:row>
+    <x:row r="257">
+      <x:c r="T257"/>
+    </x:row>
+    <x:row r="258">
+      <x:c r="T258"/>
+    </x:row>
+    <x:row r="259">
+      <x:c r="T259"/>
+    </x:row>
+    <x:row r="260">
+      <x:c r="T260"/>
+    </x:row>
+    <x:row r="261">
+      <x:c r="T261"/>
+    </x:row>
+    <x:row r="262">
+      <x:c r="T262"/>
+    </x:row>
+    <x:row r="263">
+      <x:c r="T263"/>
+    </x:row>
+    <x:row r="264">
+      <x:c r="T264"/>
+    </x:row>
+    <x:row r="265">
+      <x:c r="T265"/>
+    </x:row>
+    <x:row r="266">
+      <x:c r="T266"/>
+    </x:row>
+    <x:row r="267">
+      <x:c r="T267"/>
+    </x:row>
+    <x:row r="268">
+      <x:c r="T268"/>
+    </x:row>
+    <x:row r="269">
+      <x:c r="T269"/>
+    </x:row>
+    <x:row r="270">
+      <x:c r="T270"/>
+    </x:row>
+    <x:row r="271">
+      <x:c r="T271"/>
+    </x:row>
+    <x:row r="272">
+      <x:c r="T272"/>
+    </x:row>
+    <x:row r="273">
+      <x:c r="T273"/>
+    </x:row>
+    <x:row r="274">
+      <x:c r="T274"/>
+    </x:row>
+    <x:row r="275">
+      <x:c r="T275"/>
+    </x:row>
+    <x:row r="276">
+      <x:c r="T276"/>
+    </x:row>
+    <x:row r="277">
+      <x:c r="T277"/>
+    </x:row>
+    <x:row r="278">
+      <x:c r="T278"/>
+    </x:row>
+    <x:row r="279">
+      <x:c r="T279"/>
+    </x:row>
+    <x:row r="280">
+      <x:c r="T280"/>
+    </x:row>
+    <x:row r="281">
+      <x:c r="T281"/>
+    </x:row>
+    <x:row r="282">
+      <x:c r="T282"/>
+    </x:row>
+    <x:row r="283">
+      <x:c r="T283"/>
+    </x:row>
+    <x:row r="284">
+      <x:c r="T284"/>
+    </x:row>
+    <x:row r="285">
+      <x:c r="T285"/>
+    </x:row>
+    <x:row r="286">
+      <x:c r="T286"/>
+    </x:row>
+    <x:row r="287">
+      <x:c r="T287"/>
+    </x:row>
+    <x:row r="288">
+      <x:c r="T288"/>
+    </x:row>
+    <x:row r="289">
+      <x:c r="T289"/>
+    </x:row>
+    <x:row r="290">
+      <x:c r="T290"/>
+    </x:row>
+    <x:row r="291">
+      <x:c r="T291"/>
+    </x:row>
+    <x:row r="292">
+      <x:c r="T292"/>
+    </x:row>
+    <x:row r="293">
+      <x:c r="T293"/>
+    </x:row>
+    <x:row r="294">
+      <x:c r="T294"/>
+    </x:row>
+    <x:row r="295">
+      <x:c r="T295"/>
+    </x:row>
+    <x:row r="296">
+      <x:c r="T296"/>
+    </x:row>
+    <x:row r="297">
+      <x:c r="T297"/>
+    </x:row>
+    <x:row r="298">
+      <x:c r="T298"/>
+    </x:row>
+    <x:row r="299">
+      <x:c r="T299"/>
+    </x:row>
+    <x:row r="300">
+      <x:c r="T300"/>
+    </x:row>
+    <x:row r="301">
+      <x:c r="T301"/>
+    </x:row>
+    <x:row r="302">
+      <x:c r="T302"/>
+    </x:row>
+    <x:row r="303">
+      <x:c r="T303"/>
+    </x:row>
+    <x:row r="304">
+      <x:c r="T304"/>
+    </x:row>
+    <x:row r="305">
+      <x:c r="T305"/>
+    </x:row>
+    <x:row r="306">
+      <x:c r="T306"/>
+    </x:row>
+    <x:row r="307">
+      <x:c r="T307"/>
+    </x:row>
+    <x:row r="308">
+      <x:c r="T308"/>
+    </x:row>
+    <x:row r="309">
+      <x:c r="T309"/>
+    </x:row>
+    <x:row r="310">
+      <x:c r="T310"/>
+    </x:row>
+    <x:row r="311">
+      <x:c r="T311"/>
+    </x:row>
+    <x:row r="312">
+      <x:c r="T312"/>
+    </x:row>
+    <x:row r="313">
+      <x:c r="T313"/>
+    </x:row>
+    <x:row r="314">
+      <x:c r="T314"/>
+    </x:row>
+    <x:row r="315">
+      <x:c r="T315"/>
+    </x:row>
+    <x:row r="316">
+      <x:c r="T316"/>
+    </x:row>
+    <x:row r="317">
+      <x:c r="T317"/>
+    </x:row>
+    <x:row r="318">
+      <x:c r="T318"/>
+    </x:row>
+    <x:row r="319">
+      <x:c r="T319"/>
+    </x:row>
+    <x:row r="320">
+      <x:c r="T320"/>
+    </x:row>
+    <x:row r="321">
+      <x:c r="T321"/>
+    </x:row>
+    <x:row r="322">
+      <x:c r="T322"/>
+    </x:row>
+    <x:row r="323">
+      <x:c r="T323"/>
+    </x:row>
+    <x:row r="324">
+      <x:c r="T324"/>
+    </x:row>
+    <x:row r="325">
+      <x:c r="T325"/>
+    </x:row>
+    <x:row r="326">
+      <x:c r="T326"/>
+    </x:row>
+    <x:row r="327">
+      <x:c r="T327"/>
+    </x:row>
+    <x:row r="328">
+      <x:c r="T328"/>
+    </x:row>
+    <x:row r="329">
+      <x:c r="T329"/>
+    </x:row>
+    <x:row r="330">
+      <x:c r="T330"/>
+    </x:row>
+    <x:row r="331">
+      <x:c r="T331"/>
+    </x:row>
+    <x:row r="332">
+      <x:c r="T332"/>
+    </x:row>
+    <x:row r="333">
+      <x:c r="T333"/>
+    </x:row>
+    <x:row r="334">
+      <x:c r="T334"/>
+    </x:row>
+    <x:row r="335">
+      <x:c r="T335"/>
+    </x:row>
+    <x:row r="336">
+      <x:c r="T336"/>
+    </x:row>
+    <x:row r="337">
+      <x:c r="T337"/>
+    </x:row>
+    <x:row r="338">
+      <x:c r="T338"/>
+    </x:row>
+    <x:row r="339">
+      <x:c r="T339"/>
+    </x:row>
+    <x:row r="340">
+      <x:c r="T340"/>
+    </x:row>
+    <x:row r="341">
+      <x:c r="T341"/>
+    </x:row>
+    <x:row r="342">
+      <x:c r="T342"/>
+    </x:row>
+    <x:row r="343">
+      <x:c r="T343"/>
+    </x:row>
+    <x:row r="344">
+      <x:c r="T344"/>
+    </x:row>
+    <x:row r="345">
+      <x:c r="T345"/>
+    </x:row>
+    <x:row r="346">
+      <x:c r="T346"/>
+    </x:row>
+    <x:row r="347">
+      <x:c r="T347"/>
+    </x:row>
+    <x:row r="348">
+      <x:c r="T348"/>
+    </x:row>
+    <x:row r="349">
+      <x:c r="T349"/>
+    </x:row>
+    <x:row r="350">
+      <x:c r="T350"/>
+    </x:row>
+    <x:row r="351">
+      <x:c r="T351"/>
+    </x:row>
+    <x:row r="352">
+      <x:c r="T352"/>
+    </x:row>
+    <x:row r="353">
+      <x:c r="T353"/>
+    </x:row>
+    <x:row r="354">
+      <x:c r="T354"/>
+    </x:row>
+    <x:row r="355">
+      <x:c r="T355"/>
+    </x:row>
+    <x:row r="356">
+      <x:c r="T356"/>
+    </x:row>
+    <x:row r="357">
+      <x:c r="T357"/>
+    </x:row>
+    <x:row r="358">
+      <x:c r="T358"/>
+    </x:row>
+    <x:row r="359">
+      <x:c r="T359"/>
+    </x:row>
+    <x:row r="360">
+      <x:c r="T360"/>
+    </x:row>
+    <x:row r="361">
+      <x:c r="T361"/>
+    </x:row>
+    <x:row r="362">
+      <x:c r="T362"/>
+    </x:row>
+    <x:row r="363">
+      <x:c r="T363"/>
+    </x:row>
+    <x:row r="364">
+      <x:c r="T364"/>
+    </x:row>
+    <x:row r="365">
+      <x:c r="T365"/>
+    </x:row>
+    <x:row r="366">
+      <x:c r="T366"/>
+    </x:row>
+    <x:row r="367">
+      <x:c r="T367"/>
+    </x:row>
+    <x:row r="368">
+      <x:c r="T368"/>
+    </x:row>
+    <x:row r="369">
+      <x:c r="T369"/>
+    </x:row>
+    <x:row r="370">
+      <x:c r="T370"/>
+    </x:row>
+    <x:row r="371">
+      <x:c r="T371"/>
+    </x:row>
+    <x:row r="372">
+      <x:c r="T372"/>
+    </x:row>
+    <x:row r="373">
+      <x:c r="T373"/>
+    </x:row>
+    <x:row r="374">
+      <x:c r="T374"/>
+    </x:row>
+    <x:row r="375">
+      <x:c r="T375"/>
+    </x:row>
+    <x:row r="376">
+      <x:c r="T376"/>
+    </x:row>
+    <x:row r="377">
+      <x:c r="T377"/>
+    </x:row>
+    <x:row r="378">
+      <x:c r="T378"/>
+    </x:row>
+    <x:row r="379">
+      <x:c r="T379"/>
+    </x:row>
+    <x:row r="380">
+      <x:c r="T380"/>
+    </x:row>
+    <x:row r="381">
+      <x:c r="T381"/>
+    </x:row>
+    <x:row r="382">
+      <x:c r="T382"/>
+    </x:row>
+    <x:row r="383">
+      <x:c r="T383"/>
+    </x:row>
+    <x:row r="384">
+      <x:c r="T384"/>
+    </x:row>
+    <x:row r="385">
+      <x:c r="T385"/>
+    </x:row>
+    <x:row r="386">
+      <x:c r="T386"/>
+    </x:row>
+    <x:row r="387">
+      <x:c r="T387"/>
+    </x:row>
+    <x:row r="388">
+      <x:c r="T388"/>
+    </x:row>
+    <x:row r="389">
+      <x:c r="T389"/>
+    </x:row>
+    <x:row r="390">
+      <x:c r="T390"/>
+    </x:row>
+    <x:row r="391">
+      <x:c r="T391"/>
+    </x:row>
+    <x:row r="392">
+      <x:c r="T392"/>
+    </x:row>
+    <x:row r="393">
+      <x:c r="T393"/>
+    </x:row>
+    <x:row r="394">
+      <x:c r="T394"/>
+    </x:row>
+    <x:row r="395">
+      <x:c r="T395"/>
+    </x:row>
+    <x:row r="396">
+      <x:c r="T396"/>
+    </x:row>
+    <x:row r="397">
+      <x:c r="T397"/>
+    </x:row>
+    <x:row r="398">
+      <x:c r="T398"/>
+    </x:row>
+    <x:row r="399">
+      <x:c r="T399"/>
+    </x:row>
+    <x:row r="400">
+      <x:c r="T400"/>
+    </x:row>
+    <x:row r="401">
+      <x:c r="T401"/>
+    </x:row>
+    <x:row r="402">
+      <x:c r="T402"/>
+    </x:row>
+    <x:row r="403">
+      <x:c r="T403"/>
+    </x:row>
+    <x:row r="404">
+      <x:c r="T404"/>
+    </x:row>
+    <x:row r="405">
+      <x:c r="T405"/>
+    </x:row>
+    <x:row r="406">
+      <x:c r="T406"/>
+    </x:row>
+    <x:row r="407">
+      <x:c r="T407"/>
+    </x:row>
+    <x:row r="408">
+      <x:c r="T408"/>
+    </x:row>
+    <x:row r="409">
+      <x:c r="T409"/>
+    </x:row>
+    <x:row r="410">
+      <x:c r="T410"/>
+    </x:row>
+    <x:row r="411">
+      <x:c r="T411"/>
+    </x:row>
+    <x:row r="412">
+      <x:c r="T412"/>
+    </x:row>
+    <x:row r="413">
+      <x:c r="T413"/>
+    </x:row>
+    <x:row r="414">
+      <x:c r="T414"/>
+    </x:row>
+    <x:row r="415">
+      <x:c r="T415"/>
+    </x:row>
+    <x:row r="416">
+      <x:c r="T416"/>
+    </x:row>
+    <x:row r="417">
+      <x:c r="T417"/>
+    </x:row>
+    <x:row r="418">
+      <x:c r="T418"/>
+    </x:row>
+    <x:row r="419">
+      <x:c r="T419"/>
+    </x:row>
+    <x:row r="420">
+      <x:c r="T420"/>
+    </x:row>
+    <x:row r="421">
+      <x:c r="T421"/>
+    </x:row>
+    <x:row r="422">
+      <x:c r="T422"/>
+    </x:row>
+    <x:row r="423">
+      <x:c r="T423"/>
+    </x:row>
+    <x:row r="424">
+      <x:c r="T424"/>
+    </x:row>
+    <x:row r="425">
+      <x:c r="T425"/>
+    </x:row>
+    <x:row r="426">
+      <x:c r="T426"/>
+    </x:row>
+    <x:row r="427">
+      <x:c r="T427"/>
+    </x:row>
+    <x:row r="428">
+      <x:c r="T428"/>
+    </x:row>
+    <x:row r="429">
+      <x:c r="T429"/>
+    </x:row>
+    <x:row r="430">
+      <x:c r="T430"/>
+    </x:row>
+    <x:row r="431">
+      <x:c r="T431"/>
+    </x:row>
+    <x:row r="432">
+      <x:c r="T432"/>
+    </x:row>
+    <x:row r="433">
+      <x:c r="T433"/>
+    </x:row>
+    <x:row r="434">
+      <x:c r="T434"/>
+    </x:row>
+    <x:row r="435">
+      <x:c r="T435"/>
+    </x:row>
+    <x:row r="436">
+      <x:c r="T436"/>
+    </x:row>
+    <x:row r="437">
+      <x:c r="T437"/>
+    </x:row>
+    <x:row r="438">
+      <x:c r="T438"/>
+    </x:row>
+    <x:row r="439">
+      <x:c r="T439"/>
+    </x:row>
+    <x:row r="440">
+      <x:c r="T440"/>
+    </x:row>
+    <x:row r="441">
+      <x:c r="T441"/>
+    </x:row>
+    <x:row r="442">
+      <x:c r="T442"/>
+    </x:row>
+    <x:row r="443">
+      <x:c r="T443"/>
+    </x:row>
+    <x:row r="444">
+      <x:c r="T444"/>
+    </x:row>
+    <x:row r="445">
+      <x:c r="T445"/>
+    </x:row>
+    <x:row r="446">
+      <x:c r="T446"/>
+    </x:row>
+    <x:row r="447">
+      <x:c r="T447"/>
+    </x:row>
+    <x:row r="448">
+      <x:c r="T448"/>
+    </x:row>
+    <x:row r="449">
+      <x:c r="T449"/>
+    </x:row>
+    <x:row r="450">
+      <x:c r="T450"/>
+    </x:row>
+    <x:row r="451">
+      <x:c r="T451"/>
+    </x:row>
+    <x:row r="452">
+      <x:c r="T452"/>
+    </x:row>
+    <x:row r="453">
+      <x:c r="T453"/>
+    </x:row>
+    <x:row r="454">
+      <x:c r="T454"/>
+    </x:row>
+    <x:row r="455">
+      <x:c r="T455"/>
+    </x:row>
+    <x:row r="456">
+      <x:c r="T456"/>
+    </x:row>
+    <x:row r="457">
+      <x:c r="T457"/>
+    </x:row>
+    <x:row r="458">
+      <x:c r="T458"/>
+    </x:row>
+    <x:row r="459">
+      <x:c r="T459"/>
+    </x:row>
+    <x:row r="460">
+      <x:c r="T460"/>
+    </x:row>
+    <x:row r="461">
+      <x:c r="T461"/>
+    </x:row>
+    <x:row r="462">
+      <x:c r="T462"/>
+    </x:row>
+    <x:row r="463">
+      <x:c r="T463"/>
+    </x:row>
+    <x:row r="464">
+      <x:c r="T464"/>
+    </x:row>
+    <x:row r="465">
+      <x:c r="T465"/>
+    </x:row>
+    <x:row r="466">
+      <x:c r="T466"/>
+    </x:row>
+    <x:row r="467">
+      <x:c r="T467"/>
+    </x:row>
+    <x:row r="468">
+      <x:c r="T468"/>
+    </x:row>
+    <x:row r="469">
+      <x:c r="T469"/>
+    </x:row>
+    <x:row r="470">
+      <x:c r="T470"/>
+    </x:row>
+    <x:row r="471">
+      <x:c r="T471"/>
+    </x:row>
+    <x:row r="472">
+      <x:c r="T472"/>
+    </x:row>
+    <x:row r="473">
+      <x:c r="T473"/>
+    </x:row>
+    <x:row r="474">
+      <x:c r="T474"/>
+    </x:row>
+    <x:row r="475">
+      <x:c r="T475"/>
+    </x:row>
+    <x:row r="476">
+      <x:c r="T476"/>
+    </x:row>
+    <x:row r="477">
+      <x:c r="T477"/>
+    </x:row>
+    <x:row r="478">
+      <x:c r="T478"/>
+    </x:row>
+    <x:row r="479">
+      <x:c r="T479"/>
+    </x:row>
+    <x:row r="480">
+      <x:c r="T480"/>
+    </x:row>
+    <x:row r="481">
+      <x:c r="T481"/>
+    </x:row>
+    <x:row r="482">
+      <x:c r="T482"/>
+    </x:row>
+    <x:row r="483">
+      <x:c r="T483"/>
+    </x:row>
+    <x:row r="484">
+      <x:c r="T484"/>
+    </x:row>
+    <x:row r="485">
+      <x:c r="T485"/>
+    </x:row>
+    <x:row r="486">
+      <x:c r="T486"/>
+    </x:row>
+    <x:row r="487">
+      <x:c r="T487"/>
+    </x:row>
+    <x:row r="488">
+      <x:c r="T488"/>
+    </x:row>
+    <x:row r="489">
+      <x:c r="T489"/>
+    </x:row>
+    <x:row r="490">
+      <x:c r="T490"/>
+    </x:row>
+    <x:row r="491">
+      <x:c r="T491"/>
+    </x:row>
+    <x:row r="492">
+      <x:c r="T492"/>
+    </x:row>
+    <x:row r="493">
+      <x:c r="T493"/>
+    </x:row>
+    <x:row r="494">
+      <x:c r="T494"/>
+    </x:row>
+    <x:row r="495">
+      <x:c r="T495"/>
+    </x:row>
+    <x:row r="496">
+      <x:c r="T496"/>
+    </x:row>
+    <x:row r="497">
+      <x:c r="T497"/>
+    </x:row>
+    <x:row r="498">
+      <x:c r="T498"/>
+    </x:row>
+    <x:row r="499">
+      <x:c r="T499"/>
+    </x:row>
+    <x:row r="500">
+      <x:c r="T500"/>
+    </x:row>
+    <x:row r="501">
+      <x:c r="T501"/>
+    </x:row>
+    <x:row r="502">
+      <x:c r="T502"/>
+    </x:row>
+    <x:row r="503">
+      <x:c r="T503"/>
+    </x:row>
+    <x:row r="504">
+      <x:c r="T504"/>
+    </x:row>
+    <x:row r="505">
+      <x:c r="T505"/>
+    </x:row>
+    <x:row r="506">
+      <x:c r="T506"/>
+    </x:row>
+    <x:row r="507">
+      <x:c r="T507"/>
+    </x:row>
+    <x:row r="508">
+      <x:c r="T508"/>
+    </x:row>
+    <x:row r="509">
+      <x:c r="T509"/>
+    </x:row>
+    <x:row r="510">
+      <x:c r="T510"/>
+    </x:row>
+    <x:row r="511">
+      <x:c r="T511"/>
+    </x:row>
+    <x:row r="512">
+      <x:c r="T512"/>
+    </x:row>
+    <x:row r="513">
+      <x:c r="T513"/>
+    </x:row>
+    <x:row r="514">
+      <x:c r="T514"/>
+    </x:row>
+    <x:row r="515">
+      <x:c r="T515"/>
+    </x:row>
+    <x:row r="516">
+      <x:c r="T516"/>
+    </x:row>
+    <x:row r="517">
+      <x:c r="T517"/>
+    </x:row>
+    <x:row r="518">
+      <x:c r="T518"/>
+    </x:row>
+    <x:row r="519">
+      <x:c r="T519"/>
+    </x:row>
+    <x:row r="520">
+      <x:c r="T520"/>
+    </x:row>
+    <x:row r="521">
+      <x:c r="T521"/>
+    </x:row>
+    <x:row r="522">
+      <x:c r="T522"/>
+    </x:row>
+    <x:row r="523">
+      <x:c r="T523"/>
+    </x:row>
+    <x:row r="524">
+      <x:c r="T524"/>
+    </x:row>
+    <x:row r="525">
+      <x:c r="T525"/>
+    </x:row>
+    <x:row r="526">
+      <x:c r="T526"/>
+    </x:row>
+    <x:row r="527">
+      <x:c r="T527"/>
+    </x:row>
+    <x:row r="528">
+      <x:c r="T528"/>
+    </x:row>
+    <x:row r="529">
+      <x:c r="T529"/>
+    </x:row>
+    <x:row r="530">
+      <x:c r="T530"/>
+    </x:row>
+    <x:row r="531">
+      <x:c r="T531"/>
+    </x:row>
+    <x:row r="532">
+      <x:c r="T532"/>
+    </x:row>
+    <x:row r="533">
+      <x:c r="T533"/>
+    </x:row>
+    <x:row r="534">
+      <x:c r="T534"/>
+    </x:row>
+    <x:row r="535">
+      <x:c r="T535"/>
+    </x:row>
+    <x:row r="536">
+      <x:c r="T536"/>
+    </x:row>
+    <x:row r="537">
+      <x:c r="T537"/>
+    </x:row>
+    <x:row r="538">
+      <x:c r="T538"/>
+    </x:row>
+    <x:row r="539">
+      <x:c r="T539"/>
+    </x:row>
+    <x:row r="540">
+      <x:c r="T540"/>
+    </x:row>
+    <x:row r="541">
+      <x:c r="T541"/>
+    </x:row>
+    <x:row r="542">
+      <x:c r="T542"/>
+    </x:row>
+    <x:row r="543">
+      <x:c r="T543"/>
+    </x:row>
+    <x:row r="544">
+      <x:c r="T544"/>
+    </x:row>
+    <x:row r="545">
+      <x:c r="T545"/>
+    </x:row>
+    <x:row r="546">
+      <x:c r="T546"/>
+    </x:row>
+    <x:row r="547">
+      <x:c r="T547"/>
+    </x:row>
+    <x:row r="548">
+      <x:c r="T548"/>
+    </x:row>
+    <x:row r="549">
+      <x:c r="T549"/>
+    </x:row>
+    <x:row r="550">
+      <x:c r="T550"/>
+    </x:row>
+    <x:row r="551">
+      <x:c r="T551"/>
+    </x:row>
+    <x:row r="552">
+      <x:c r="T552"/>
+    </x:row>
+    <x:row r="553">
+      <x:c r="T553"/>
+    </x:row>
+    <x:row r="554">
+      <x:c r="T554"/>
+    </x:row>
+    <x:row r="555">
+      <x:c r="T555"/>
+    </x:row>
+    <x:row r="556">
+      <x:c r="T556"/>
+    </x:row>
+    <x:row r="557">
+      <x:c r="T557"/>
+    </x:row>
+    <x:row r="558">
+      <x:c r="T558"/>
+    </x:row>
+    <x:row r="559">
+      <x:c r="T559"/>
+    </x:row>
+    <x:row r="560">
+      <x:c r="T560"/>
+    </x:row>
+    <x:row r="561">
+      <x:c r="T561"/>
+    </x:row>
+    <x:row r="562">
+      <x:c r="T562"/>
+    </x:row>
+    <x:row r="563">
+      <x:c r="T563"/>
+    </x:row>
+    <x:row r="564">
+      <x:c r="T564"/>
+    </x:row>
+    <x:row r="565">
+      <x:c r="T565"/>
+    </x:row>
+    <x:row r="566">
+      <x:c r="T566"/>
+    </x:row>
+    <x:row r="567">
+      <x:c r="T567"/>
+    </x:row>
+    <x:row r="568">
+      <x:c r="T568"/>
+    </x:row>
+    <x:row r="569">
+      <x:c r="T569"/>
+    </x:row>
+    <x:row r="570">
+      <x:c r="T570"/>
+    </x:row>
+    <x:row r="571">
+      <x:c r="T571"/>
+    </x:row>
+    <x:row r="572">
+      <x:c r="T572"/>
+    </x:row>
+    <x:row r="573">
+      <x:c r="T573"/>
+    </x:row>
+    <x:row r="574">
+      <x:c r="T574"/>
+    </x:row>
+    <x:row r="575">
+      <x:c r="T575"/>
+    </x:row>
+    <x:row r="576">
+      <x:c r="T576"/>
+    </x:row>
+    <x:row r="577">
+      <x:c r="T577"/>
+    </x:row>
+    <x:row r="578">
+      <x:c r="T578"/>
+    </x:row>
+    <x:row r="579">
+      <x:c r="T579"/>
+    </x:row>
+    <x:row r="580">
+      <x:c r="T580"/>
+    </x:row>
+    <x:row r="581">
+      <x:c r="T581"/>
+    </x:row>
+    <x:row r="582">
+      <x:c r="T582"/>
+    </x:row>
+    <x:row r="583">
+      <x:c r="T583"/>
+    </x:row>
+    <x:row r="584">
+      <x:c r="T584"/>
+    </x:row>
+    <x:row r="585">
+      <x:c r="T585"/>
+    </x:row>
+    <x:row r="586">
+      <x:c r="T586"/>
+    </x:row>
+    <x:row r="587">
+      <x:c r="T587"/>
+    </x:row>
+    <x:row r="588">
+      <x:c r="T588"/>
+    </x:row>
+    <x:row r="589">
+      <x:c r="T589"/>
+    </x:row>
+    <x:row r="590">
+      <x:c r="T590"/>
+    </x:row>
+    <x:row r="591">
+      <x:c r="T591"/>
+    </x:row>
+    <x:row r="592">
+      <x:c r="T592"/>
+    </x:row>
+    <x:row r="593">
+      <x:c r="T593"/>
+    </x:row>
+    <x:row r="594">
+      <x:c r="T594"/>
+    </x:row>
+    <x:row r="595">
+      <x:c r="T595"/>
+    </x:row>
+    <x:row r="596">
+      <x:c r="T596"/>
+    </x:row>
+    <x:row r="597">
+      <x:c r="T597"/>
+    </x:row>
+    <x:row r="598">
+      <x:c r="T598"/>
+    </x:row>
+    <x:row r="599">
+      <x:c r="T599"/>
+    </x:row>
+    <x:row r="600">
+      <x:c r="T600"/>
+    </x:row>
+    <x:row r="601">
+      <x:c r="T601"/>
+    </x:row>
+    <x:row r="602">
+      <x:c r="T602"/>
+    </x:row>
+    <x:row r="603">
+      <x:c r="T603"/>
+    </x:row>
+    <x:row r="604">
+      <x:c r="T604"/>
+    </x:row>
+    <x:row r="605">
+      <x:c r="T605"/>
+    </x:row>
+    <x:row r="606">
+      <x:c r="T606"/>
+    </x:row>
+    <x:row r="607">
+      <x:c r="T607"/>
+    </x:row>
+    <x:row r="608">
+      <x:c r="T608"/>
+    </x:row>
+    <x:row r="609">
+      <x:c r="T609"/>
+    </x:row>
+    <x:row r="610">
+      <x:c r="T610"/>
+    </x:row>
+    <x:row r="611">
+      <x:c r="T611"/>
+    </x:row>
+    <x:row r="612">
+      <x:c r="T612"/>
+    </x:row>
+    <x:row r="613">
+      <x:c r="T613"/>
+    </x:row>
+    <x:row r="614">
+      <x:c r="T614"/>
+    </x:row>
+    <x:row r="615">
+      <x:c r="T615"/>
+    </x:row>
+    <x:row r="616">
+      <x:c r="T616"/>
+    </x:row>
+    <x:row r="617">
+      <x:c r="T617"/>
+    </x:row>
+    <x:row r="618">
+      <x:c r="T618"/>
+    </x:row>
+    <x:row r="619">
+      <x:c r="T619"/>
+    </x:row>
+    <x:row r="620">
+      <x:c r="T620"/>
+    </x:row>
+    <x:row r="621">
+      <x:c r="T621"/>
+    </x:row>
+    <x:row r="622">
+      <x:c r="T622"/>
+    </x:row>
+    <x:row r="623">
+      <x:c r="T623"/>
+    </x:row>
+    <x:row r="624">
+      <x:c r="T624"/>
+    </x:row>
+    <x:row r="625">
+      <x:c r="T625"/>
+    </x:row>
+    <x:row r="626">
+      <x:c r="T626"/>
+    </x:row>
+    <x:row r="627">
+      <x:c r="T627"/>
+    </x:row>
+    <x:row r="628">
+      <x:c r="T628"/>
+    </x:row>
+    <x:row r="629">
+      <x:c r="T629"/>
+    </x:row>
+    <x:row r="630">
+      <x:c r="T630"/>
+    </x:row>
+    <x:row r="631">
+      <x:c r="T631"/>
+    </x:row>
+    <x:row r="632">
+      <x:c r="T632"/>
+    </x:row>
+    <x:row r="633">
+      <x:c r="T633"/>
+    </x:row>
+    <x:row r="634">
+      <x:c r="T634"/>
+    </x:row>
+    <x:row r="635">
+      <x:c r="T635"/>
+    </x:row>
+    <x:row r="636">
+      <x:c r="T636"/>
+    </x:row>
+    <x:row r="637">
+      <x:c r="T637"/>
+    </x:row>
+    <x:row r="638">
+      <x:c r="T638"/>
+    </x:row>
+    <x:row r="639">
+      <x:c r="T639"/>
+    </x:row>
+    <x:row r="640">
+      <x:c r="T640"/>
+    </x:row>
+    <x:row r="641">
+      <x:c r="T641"/>
+    </x:row>
+    <x:row r="642">
+      <x:c r="T642"/>
+    </x:row>
+    <x:row r="643">
+      <x:c r="T643"/>
+    </x:row>
+    <x:row r="644">
+      <x:c r="T644"/>
+    </x:row>
+    <x:row r="645">
+      <x:c r="T645"/>
+    </x:row>
+    <x:row r="646">
+      <x:c r="T646"/>
+    </x:row>
+    <x:row r="647">
+      <x:c r="T647"/>
+    </x:row>
+    <x:row r="648">
+      <x:c r="T648"/>
+    </x:row>
+    <x:row r="649">
+      <x:c r="T649"/>
+    </x:row>
+    <x:row r="650">
+      <x:c r="T650"/>
+    </x:row>
+    <x:row r="651">
+      <x:c r="T651"/>
+    </x:row>
+    <x:row r="652">
+      <x:c r="T652"/>
+    </x:row>
+    <x:row r="653">
+      <x:c r="T653"/>
+    </x:row>
+    <x:row r="654">
+      <x:c r="T654"/>
+    </x:row>
+    <x:row r="655">
+      <x:c r="T655"/>
+    </x:row>
+    <x:row r="656">
+      <x:c r="T656"/>
+    </x:row>
+    <x:row r="657">
+      <x:c r="T657"/>
+    </x:row>
+    <x:row r="658">
+      <x:c r="T658"/>
+    </x:row>
+    <x:row r="659">
+      <x:c r="T659"/>
+    </x:row>
+    <x:row r="660">
+      <x:c r="T660"/>
+    </x:row>
+    <x:row r="661">
+      <x:c r="T661"/>
+    </x:row>
+    <x:row r="662">
+      <x:c r="T662"/>
+    </x:row>
+    <x:row r="663">
+      <x:c r="T663"/>
+    </x:row>
+    <x:row r="664">
+      <x:c r="T664"/>
+    </x:row>
+    <x:row r="665">
+      <x:c r="T665"/>
+    </x:row>
+    <x:row r="666">
+      <x:c r="T666"/>
+    </x:row>
+    <x:row r="667">
+      <x:c r="T667"/>
+    </x:row>
+    <x:row r="668">
+      <x:c r="T668"/>
+    </x:row>
+    <x:row r="669">
+      <x:c r="T669"/>
+    </x:row>
+    <x:row r="670">
+      <x:c r="T670"/>
+    </x:row>
+    <x:row r="671">
+      <x:c r="T671"/>
+    </x:row>
+    <x:row r="672">
+      <x:c r="T672"/>
+    </x:row>
+    <x:row r="673">
+      <x:c r="T673"/>
+    </x:row>
+    <x:row r="674">
+      <x:c r="T674"/>
+    </x:row>
+    <x:row r="675">
+      <x:c r="T675"/>
+    </x:row>
+    <x:row r="676">
+      <x:c r="T676"/>
+    </x:row>
+    <x:row r="677">
+      <x:c r="T677"/>
+    </x:row>
+    <x:row r="678">
+      <x:c r="T678"/>
+    </x:row>
+    <x:row r="679">
+      <x:c r="T679"/>
+    </x:row>
+    <x:row r="680">
+      <x:c r="T680"/>
+    </x:row>
+    <x:row r="681">
+      <x:c r="T681"/>
+    </x:row>
+    <x:row r="682">
+      <x:c r="T682"/>
+    </x:row>
+    <x:row r="683">
+      <x:c r="T683"/>
+    </x:row>
+    <x:row r="684">
+      <x:c r="T684"/>
+    </x:row>
+    <x:row r="685">
+      <x:c r="T685"/>
+    </x:row>
+    <x:row r="686">
+      <x:c r="T686"/>
+    </x:row>
+    <x:row r="687">
+      <x:c r="T687"/>
+    </x:row>
+    <x:row r="688">
+      <x:c r="T688"/>
+    </x:row>
+    <x:row r="689">
+      <x:c r="T689"/>
+    </x:row>
+    <x:row r="690">
+      <x:c r="T690"/>
+    </x:row>
+    <x:row r="691">
+      <x:c r="T691"/>
+    </x:row>
+    <x:row r="692">
+      <x:c r="T692"/>
+    </x:row>
+    <x:row r="693">
+      <x:c r="T693"/>
+    </x:row>
+    <x:row r="694">
+      <x:c r="T694"/>
+    </x:row>
+    <x:row r="695">
+      <x:c r="T695"/>
+    </x:row>
+    <x:row r="696">
+      <x:c r="T696"/>
+    </x:row>
+    <x:row r="697">
+      <x:c r="T697"/>
+    </x:row>
+    <x:row r="698">
+      <x:c r="T698"/>
+    </x:row>
+    <x:row r="699">
+      <x:c r="T699"/>
+    </x:row>
+    <x:row r="700">
+      <x:c r="T700"/>
+    </x:row>
+    <x:row r="701">
+      <x:c r="T701"/>
+    </x:row>
+    <x:row r="702">
+      <x:c r="T702"/>
+    </x:row>
+    <x:row r="703">
+      <x:c r="T703"/>
+    </x:row>
+    <x:row r="704">
+      <x:c r="T704"/>
+    </x:row>
+    <x:row r="705">
+      <x:c r="T705"/>
+    </x:row>
+    <x:row r="706">
+      <x:c r="T706"/>
+    </x:row>
+    <x:row r="707">
+      <x:c r="T707"/>
+    </x:row>
+    <x:row r="708">
+      <x:c r="T708"/>
+    </x:row>
+    <x:row r="709">
+      <x:c r="T709"/>
+    </x:row>
+    <x:row r="710">
+      <x:c r="T710"/>
+    </x:row>
+    <x:row r="711">
+      <x:c r="T711"/>
+    </x:row>
+    <x:row r="712">
+      <x:c r="T712"/>
+    </x:row>
+    <x:row r="713">
+      <x:c r="T713"/>
+    </x:row>
+    <x:row r="714">
+      <x:c r="T714"/>
+    </x:row>
+    <x:row r="715">
+      <x:c r="T715"/>
+    </x:row>
+    <x:row r="716">
+      <x:c r="T716"/>
+    </x:row>
+    <x:row r="717">
+      <x:c r="T717"/>
+    </x:row>
+    <x:row r="718">
+      <x:c r="T718"/>
+    </x:row>
+    <x:row r="719">
+      <x:c r="T719"/>
+    </x:row>
+    <x:row r="720">
+      <x:c r="T720"/>
+    </x:row>
+    <x:row r="721">
+      <x:c r="T721"/>
+    </x:row>
+    <x:row r="722">
+      <x:c r="T722"/>
+    </x:row>
+    <x:row r="723">
+      <x:c r="T723"/>
+    </x:row>
+    <x:row r="724">
+      <x:c r="T724"/>
+    </x:row>
+    <x:row r="725">
+      <x:c r="T725"/>
+    </x:row>
+    <x:row r="726">
+      <x:c r="T726"/>
+    </x:row>
+    <x:row r="727">
+      <x:c r="T727"/>
+    </x:row>
+    <x:row r="728">
+      <x:c r="T728"/>
+    </x:row>
+    <x:row r="729">
+      <x:c r="T729"/>
+    </x:row>
+    <x:row r="730">
+      <x:c r="T730"/>
+    </x:row>
+    <x:row r="731">
+      <x:c r="T731"/>
+    </x:row>
+    <x:row r="732">
+      <x:c r="T732"/>
+    </x:row>
+    <x:row r="733">
+      <x:c r="T733"/>
+    </x:row>
+    <x:row r="734">
+      <x:c r="T734"/>
+    </x:row>
+    <x:row r="735">
+      <x:c r="T735"/>
+    </x:row>
+    <x:row r="736">
+      <x:c r="T736"/>
+    </x:row>
+    <x:row r="737">
+      <x:c r="T737"/>
+    </x:row>
+    <x:row r="738">
+      <x:c r="T738"/>
+    </x:row>
+    <x:row r="739">
+      <x:c r="T739"/>
+    </x:row>
+    <x:row r="740">
+      <x:c r="T740"/>
+    </x:row>
+    <x:row r="741">
+      <x:c r="T741"/>
+    </x:row>
+    <x:row r="742">
+      <x:c r="T742"/>
+    </x:row>
+    <x:row r="743">
+      <x:c r="T743"/>
+    </x:row>
+    <x:row r="744">
+      <x:c r="T744"/>
+    </x:row>
+    <x:row r="745">
+      <x:c r="T745"/>
+    </x:row>
+    <x:row r="746">
+      <x:c r="T746"/>
+    </x:row>
+    <x:row r="747">
+      <x:c r="T747"/>
+    </x:row>
+    <x:row r="748">
+      <x:c r="T748"/>
+    </x:row>
+    <x:row r="749">
+      <x:c r="T749"/>
+    </x:row>
+    <x:row r="750">
+      <x:c r="T750"/>
+    </x:row>
+    <x:row r="751">
+      <x:c r="T751"/>
+    </x:row>
+    <x:row r="752">
+      <x:c r="T752"/>
+    </x:row>
+    <x:row r="753">
+      <x:c r="T753"/>
+    </x:row>
+    <x:row r="754">
+      <x:c r="T754"/>
+    </x:row>
+    <x:row r="755">
+      <x:c r="T755"/>
+    </x:row>
+    <x:row r="756">
+      <x:c r="T756"/>
+    </x:row>
+    <x:row r="757">
+      <x:c r="T757"/>
+    </x:row>
+    <x:row r="758">
+      <x:c r="T758"/>
+    </x:row>
+    <x:row r="759">
+      <x:c r="T759"/>
+    </x:row>
+    <x:row r="760">
+      <x:c r="T760"/>
+    </x:row>
+    <x:row r="761">
+      <x:c r="T761"/>
+    </x:row>
+    <x:row r="762">
+      <x:c r="T762"/>
+    </x:row>
+    <x:row r="763">
+      <x:c r="T763"/>
+    </x:row>
+    <x:row r="764">
+      <x:c r="T764"/>
+    </x:row>
+    <x:row r="765">
+      <x:c r="T765"/>
+    </x:row>
+    <x:row r="766">
+      <x:c r="T766"/>
+    </x:row>
+    <x:row r="767">
+      <x:c r="T767"/>
+    </x:row>
+    <x:row r="768">
+      <x:c r="T768"/>
+    </x:row>
+    <x:row r="769">
+      <x:c r="T769"/>
+    </x:row>
+    <x:row r="770">
+      <x:c r="T770"/>
+    </x:row>
+    <x:row r="771">
+      <x:c r="T771"/>
+    </x:row>
+    <x:row r="772">
+      <x:c r="T772"/>
+    </x:row>
+    <x:row r="773">
+      <x:c r="T773"/>
+    </x:row>
+    <x:row r="774">
+      <x:c r="T774"/>
+    </x:row>
+    <x:row r="775">
+      <x:c r="T775"/>
+    </x:row>
+    <x:row r="776">
+      <x:c r="T776"/>
+    </x:row>
+    <x:row r="777">
+      <x:c r="T777"/>
+    </x:row>
+    <x:row r="778">
+      <x:c r="T778"/>
+    </x:row>
+    <x:row r="779">
+      <x:c r="T779"/>
+    </x:row>
+    <x:row r="780">
+      <x:c r="T780"/>
+    </x:row>
+    <x:row r="781">
+      <x:c r="T781"/>
+    </x:row>
+    <x:row r="782">
+      <x:c r="T782"/>
+    </x:row>
+    <x:row r="783">
+      <x:c r="T783"/>
+    </x:row>
+    <x:row r="784">
+      <x:c r="T784"/>
+    </x:row>
+    <x:row r="785">
+      <x:c r="T785"/>
+    </x:row>
+    <x:row r="786">
+      <x:c r="T786"/>
+    </x:row>
+    <x:row r="787">
+      <x:c r="T787"/>
+    </x:row>
+    <x:row r="788">
+      <x:c r="T788"/>
+    </x:row>
+    <x:row r="789">
+      <x:c r="T789"/>
+    </x:row>
+    <x:row r="790">
+      <x:c r="T790"/>
+    </x:row>
+    <x:row r="791">
+      <x:c r="T791"/>
+    </x:row>
+    <x:row r="792">
+      <x:c r="T792"/>
+    </x:row>
+    <x:row r="793">
+      <x:c r="T793"/>
+    </x:row>
+    <x:row r="794">
+      <x:c r="T794"/>
+    </x:row>
+    <x:row r="795">
+      <x:c r="T795"/>
+    </x:row>
+    <x:row r="796">
+      <x:c r="T796"/>
+    </x:row>
+    <x:row r="797">
+      <x:c r="T797"/>
+    </x:row>
+    <x:row r="798">
+      <x:c r="T798"/>
+    </x:row>
+    <x:row r="799">
+      <x:c r="T799"/>
+    </x:row>
+    <x:row r="800">
+      <x:c r="T800"/>
+    </x:row>
+    <x:row r="801">
+      <x:c r="T801"/>
+    </x:row>
+    <x:row r="802">
+      <x:c r="T802"/>
+    </x:row>
+    <x:row r="803">
+      <x:c r="T803"/>
+    </x:row>
+    <x:row r="804">
+      <x:c r="T804"/>
+    </x:row>
+    <x:row r="805">
+      <x:c r="T805"/>
+    </x:row>
+    <x:row r="806">
+      <x:c r="T806"/>
+    </x:row>
+    <x:row r="807">
+      <x:c r="T807"/>
+    </x:row>
+    <x:row r="808">
+      <x:c r="T808"/>
+    </x:row>
+    <x:row r="809">
+      <x:c r="T809"/>
+    </x:row>
+    <x:row r="810">
+      <x:c r="T810"/>
+    </x:row>
+    <x:row r="811">
+      <x:c r="T811"/>
+    </x:row>
+    <x:row r="812">
+      <x:c r="T812"/>
+    </x:row>
+    <x:row r="813">
+      <x:c r="T813"/>
+    </x:row>
+    <x:row r="814">
+      <x:c r="T814"/>
+    </x:row>
+    <x:row r="815">
+      <x:c r="T815"/>
+    </x:row>
+    <x:row r="816">
+      <x:c r="T816"/>
+    </x:row>
+    <x:row r="817">
+      <x:c r="T817"/>
+    </x:row>
+    <x:row r="818">
+      <x:c r="T818"/>
+    </x:row>
+    <x:row r="819">
+      <x:c r="T819"/>
+    </x:row>
+    <x:row r="820">
+      <x:c r="T820"/>
+    </x:row>
+    <x:row r="821">
+      <x:c r="T821"/>
+    </x:row>
+    <x:row r="822">
+      <x:c r="T822"/>
+    </x:row>
+    <x:row r="823">
+      <x:c r="T823"/>
+    </x:row>
+    <x:row r="824">
+      <x:c r="T824"/>
+    </x:row>
+    <x:row r="825">
+      <x:c r="T825"/>
+    </x:row>
+    <x:row r="826">
+      <x:c r="T826"/>
+    </x:row>
+    <x:row r="827">
+      <x:c r="T827"/>
+    </x:row>
+    <x:row r="828">
+      <x:c r="T828"/>
+    </x:row>
+    <x:row r="829">
+      <x:c r="T829"/>
+    </x:row>
+    <x:row r="830">
+      <x:c r="T830"/>
+    </x:row>
+    <x:row r="831">
+      <x:c r="T831"/>
+    </x:row>
+    <x:row r="832">
+      <x:c r="T832"/>
+    </x:row>
+    <x:row r="833">
+      <x:c r="T833"/>
+    </x:row>
+    <x:row r="834">
+      <x:c r="T834"/>
+    </x:row>
+    <x:row r="835">
+      <x:c r="T835"/>
+    </x:row>
+    <x:row r="836">
+      <x:c r="T836"/>
+    </x:row>
+    <x:row r="837">
+      <x:c r="T837"/>
+    </x:row>
+    <x:row r="838">
+      <x:c r="T838"/>
+    </x:row>
+    <x:row r="839">
+      <x:c r="T839"/>
+    </x:row>
+    <x:row r="840">
+      <x:c r="T840"/>
+    </x:row>
+    <x:row r="841">
+      <x:c r="T841"/>
+    </x:row>
+    <x:row r="842">
+      <x:c r="T842"/>
+    </x:row>
+    <x:row r="843">
+      <x:c r="T843"/>
+    </x:row>
+    <x:row r="844">
+      <x:c r="T844"/>
+    </x:row>
+    <x:row r="845">
+      <x:c r="T845"/>
+    </x:row>
+    <x:row r="846">
+      <x:c r="T846"/>
+    </x:row>
+    <x:row r="847">
+      <x:c r="T847"/>
+    </x:row>
+    <x:row r="848">
+      <x:c r="T848"/>
+    </x:row>
+    <x:row r="849">
+      <x:c r="T849"/>
+    </x:row>
+    <x:row r="850">
+      <x:c r="T850"/>
+    </x:row>
+    <x:row r="851">
+      <x:c r="T851"/>
+    </x:row>
+    <x:row r="852">
+      <x:c r="T852"/>
+    </x:row>
+    <x:row r="853">
+      <x:c r="T853"/>
+    </x:row>
+    <x:row r="854">
+      <x:c r="T854"/>
+    </x:row>
+    <x:row r="855">
+      <x:c r="T855"/>
+    </x:row>
+    <x:row r="856">
+      <x:c r="T856"/>
+    </x:row>
+    <x:row r="857">
+      <x:c r="T857"/>
+    </x:row>
+    <x:row r="858">
+      <x:c r="T858"/>
+    </x:row>
+    <x:row r="859">
+      <x:c r="T859"/>
+    </x:row>
+    <x:row r="860">
+      <x:c r="T860"/>
+    </x:row>
+    <x:row r="861">
+      <x:c r="T861"/>
+    </x:row>
+    <x:row r="862">
+      <x:c r="T862"/>
+    </x:row>
+    <x:row r="863">
+      <x:c r="T863"/>
+    </x:row>
+    <x:row r="864">
+      <x:c r="T864"/>
+    </x:row>
+    <x:row r="865">
+      <x:c r="T865"/>
+    </x:row>
+    <x:row r="866">
+      <x:c r="T866"/>
+    </x:row>
+    <x:row r="867">
+      <x:c r="T867"/>
+    </x:row>
+    <x:row r="868">
+      <x:c r="T868"/>
+    </x:row>
+    <x:row r="869">
+      <x:c r="T869"/>
+    </x:row>
+    <x:row r="870">
+      <x:c r="T870"/>
+    </x:row>
+    <x:row r="871">
+      <x:c r="T871"/>
+    </x:row>
+    <x:row r="872">
+      <x:c r="T872"/>
+    </x:row>
+    <x:row r="873">
+      <x:c r="T873"/>
+    </x:row>
+    <x:row r="874">
+      <x:c r="T874"/>
+    </x:row>
+    <x:row r="875">
+      <x:c r="T875"/>
+    </x:row>
+    <x:row r="876">
+      <x:c r="T876"/>
+    </x:row>
+    <x:row r="877">
+      <x:c r="T877"/>
+    </x:row>
+    <x:row r="878">
+      <x:c r="T878"/>
+    </x:row>
+    <x:row r="879">
+      <x:c r="T879"/>
+    </x:row>
+    <x:row r="880">
+      <x:c r="T880"/>
+    </x:row>
+    <x:row r="881">
+      <x:c r="T881"/>
+    </x:row>
+    <x:row r="882">
+      <x:c r="T882"/>
+    </x:row>
+    <x:row r="883">
+      <x:c r="T883"/>
+    </x:row>
+    <x:row r="884">
+      <x:c r="T884"/>
+    </x:row>
+    <x:row r="885">
+      <x:c r="T885"/>
+    </x:row>
+    <x:row r="886">
+      <x:c r="T886"/>
+    </x:row>
+    <x:row r="887">
+      <x:c r="T887"/>
+    </x:row>
+    <x:row r="888">
+      <x:c r="T888"/>
+    </x:row>
+    <x:row r="889">
+      <x:c r="T889"/>
+    </x:row>
+    <x:row r="890">
+      <x:c r="T890"/>
+    </x:row>
+    <x:row r="891">
+      <x:c r="T891"/>
+    </x:row>
+    <x:row r="892">
+      <x:c r="T892"/>
+    </x:row>
+    <x:row r="893">
+      <x:c r="T893"/>
+    </x:row>
+    <x:row r="894">
+      <x:c r="T894"/>
+    </x:row>
+    <x:row r="895">
+      <x:c r="T895"/>
+    </x:row>
+    <x:row r="896">
+      <x:c r="T896"/>
+    </x:row>
+    <x:row r="897">
+      <x:c r="T897"/>
+    </x:row>
+    <x:row r="898">
+      <x:c r="T898"/>
+    </x:row>
+    <x:row r="899">
+      <x:c r="T899"/>
+    </x:row>
+    <x:row r="900">
+      <x:c r="T900"/>
+    </x:row>
+    <x:row r="901">
+      <x:c r="T901"/>
+    </x:row>
+    <x:row r="902">
+      <x:c r="T902"/>
+    </x:row>
+    <x:row r="903">
+      <x:c r="T903"/>
+    </x:row>
+    <x:row r="904">
+      <x:c r="T904"/>
+    </x:row>
+    <x:row r="905">
+      <x:c r="T905"/>
+    </x:row>
+    <x:row r="906">
+      <x:c r="T906"/>
+    </x:row>
+    <x:row r="907">
+      <x:c r="T907"/>
+    </x:row>
+    <x:row r="908">
+      <x:c r="T908"/>
+    </x:row>
+    <x:row r="909">
+      <x:c r="T909"/>
+    </x:row>
+    <x:row r="910">
+      <x:c r="T910"/>
+    </x:row>
+    <x:row r="911">
+      <x:c r="T911"/>
+    </x:row>
+    <x:row r="912">
+      <x:c r="T912"/>
+    </x:row>
+    <x:row r="913">
+      <x:c r="T913"/>
+    </x:row>
+    <x:row r="914">
+      <x:c r="T914"/>
+    </x:row>
+    <x:row r="915">
+      <x:c r="T915"/>
+    </x:row>
+    <x:row r="916">
+      <x:c r="T916"/>
+    </x:row>
+    <x:row r="917">
+      <x:c r="T917"/>
+    </x:row>
+    <x:row r="918">
+      <x:c r="T918"/>
+    </x:row>
+    <x:row r="919">
+      <x:c r="T919"/>
+    </x:row>
+    <x:row r="920">
+      <x:c r="T920"/>
+    </x:row>
+    <x:row r="921">
+      <x:c r="T921"/>
+    </x:row>
+    <x:row r="922">
+      <x:c r="T922"/>
+    </x:row>
+    <x:row r="923">
+      <x:c r="T923"/>
+    </x:row>
+    <x:row r="924">
+      <x:c r="T924"/>
+    </x:row>
+    <x:row r="925">
+      <x:c r="T925"/>
+    </x:row>
+    <x:row r="926">
+      <x:c r="T926"/>
+    </x:row>
+    <x:row r="927">
+      <x:c r="T927"/>
+    </x:row>
+    <x:row r="928">
+      <x:c r="T928"/>
+    </x:row>
+    <x:row r="929">
+      <x:c r="T929"/>
+    </x:row>
+    <x:row r="930">
+      <x:c r="T930"/>
+    </x:row>
+    <x:row r="931">
+      <x:c r="T931"/>
+    </x:row>
+    <x:row r="932">
+      <x:c r="T932"/>
+    </x:row>
+    <x:row r="933">
+      <x:c r="T933"/>
+    </x:row>
+    <x:row r="934">
+      <x:c r="T934"/>
+    </x:row>
+    <x:row r="935">
+      <x:c r="T935"/>
+    </x:row>
+    <x:row r="936">
+      <x:c r="T936"/>
+    </x:row>
+    <x:row r="937">
+      <x:c r="T937"/>
+    </x:row>
+    <x:row r="938">
+      <x:c r="T938"/>
+    </x:row>
+    <x:row r="939">
+      <x:c r="T939"/>
+    </x:row>
+    <x:row r="940">
+      <x:c r="T940"/>
+    </x:row>
+    <x:row r="941">
+      <x:c r="T941"/>
+    </x:row>
+    <x:row r="942">
+      <x:c r="T942"/>
+    </x:row>
+    <x:row r="943">
+      <x:c r="T943"/>
+    </x:row>
+    <x:row r="944">
+      <x:c r="T944"/>
+    </x:row>
+    <x:row r="945">
+      <x:c r="T945"/>
+    </x:row>
+    <x:row r="946">
+      <x:c r="T946"/>
+    </x:row>
+    <x:row r="947">
+      <x:c r="T947"/>
+    </x:row>
+    <x:row r="948">
+      <x:c r="T948"/>
+    </x:row>
+    <x:row r="949">
+      <x:c r="T949"/>
+    </x:row>
+    <x:row r="950">
+      <x:c r="T950"/>
+    </x:row>
+    <x:row r="951">
+      <x:c r="T951"/>
+    </x:row>
+    <x:row r="952">
+      <x:c r="T952"/>
+    </x:row>
+    <x:row r="953">
+      <x:c r="T953"/>
+    </x:row>
+    <x:row r="954">
+      <x:c r="T954"/>
+    </x:row>
+    <x:row r="955">
+      <x:c r="T955"/>
+    </x:row>
+    <x:row r="956">
+      <x:c r="T956"/>
+    </x:row>
+    <x:row r="957">
+      <x:c r="T957"/>
+    </x:row>
+    <x:row r="958">
+      <x:c r="T958"/>
+    </x:row>
+    <x:row r="959">
+      <x:c r="T959"/>
+    </x:row>
+    <x:row r="960">
+      <x:c r="T960"/>
+    </x:row>
+    <x:row r="961">
+      <x:c r="T961"/>
+    </x:row>
+    <x:row r="962">
+      <x:c r="T962"/>
+    </x:row>
+    <x:row r="963">
+      <x:c r="T963"/>
+    </x:row>
+    <x:row r="964">
+      <x:c r="T964"/>
+    </x:row>
+    <x:row r="965">
+      <x:c r="T965"/>
+    </x:row>
+    <x:row r="966">
+      <x:c r="T966"/>
+    </x:row>
+    <x:row r="967">
+      <x:c r="T967"/>
+    </x:row>
+    <x:row r="968">
+      <x:c r="T968"/>
+    </x:row>
+    <x:row r="969">
+      <x:c r="T969"/>
+    </x:row>
+    <x:row r="970">
+      <x:c r="T970"/>
+    </x:row>
+    <x:row r="971">
+      <x:c r="T971"/>
+    </x:row>
+    <x:row r="972">
+      <x:c r="T972"/>
+    </x:row>
+    <x:row r="973">
+      <x:c r="T973"/>
+    </x:row>
+    <x:row r="974">
+      <x:c r="T974"/>
+    </x:row>
+    <x:row r="975">
+      <x:c r="T975"/>
+    </x:row>
+    <x:row r="976">
+      <x:c r="T976"/>
+    </x:row>
+    <x:row r="977">
+      <x:c r="T977"/>
+    </x:row>
+    <x:row r="978">
+      <x:c r="T978"/>
+    </x:row>
+    <x:row r="979">
+      <x:c r="T979"/>
+    </x:row>
+    <x:row r="980">
+      <x:c r="T980"/>
+    </x:row>
+    <x:row r="981">
+      <x:c r="T981"/>
+    </x:row>
+    <x:row r="982">
+      <x:c r="T982"/>
+    </x:row>
+    <x:row r="983">
+      <x:c r="T983"/>
+    </x:row>
+    <x:row r="984">
+      <x:c r="T984"/>
+    </x:row>
+    <x:row r="985">
+      <x:c r="T985"/>
+    </x:row>
+    <x:row r="986">
+      <x:c r="T986"/>
+    </x:row>
+    <x:row r="987">
+      <x:c r="T987"/>
+    </x:row>
+    <x:row r="988">
+      <x:c r="T988"/>
+    </x:row>
+    <x:row r="989">
+      <x:c r="T989"/>
+    </x:row>
+    <x:row r="990">
+      <x:c r="T990"/>
+    </x:row>
+    <x:row r="991">
+      <x:c r="T991"/>
+    </x:row>
+    <x:row r="992">
+      <x:c r="T992"/>
+    </x:row>
+    <x:row r="993">
+      <x:c r="T993"/>
+    </x:row>
+    <x:row r="994">
+      <x:c r="T994"/>
+    </x:row>
+    <x:row r="995">
+      <x:c r="T995"/>
+    </x:row>
+    <x:row r="996">
+      <x:c r="T996"/>
+    </x:row>
+    <x:row r="997">
+      <x:c r="T997"/>
+    </x:row>
+    <x:row r="998">
+      <x:c r="T998"/>
+    </x:row>
+    <x:row r="999">
+      <x:c r="T999"/>
+    </x:row>
+    <x:row r="1000">
+      <x:c r="T1000"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1462,7 +4253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96e61c61b89348ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73a05fa7333740ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3780,7 +6571,7 @@
         <x:v>schema_version</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>0.8</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>入力契約バージョン</x:v>

</xml_diff>

<commit_message>
Add decomposed solving and flexible campus transfers
</commit_message>
<xml_diff>
--- a/projects/sample/input/時間割入力_サンプル.xlsx
+++ b/projects/sample/input/時間割入力_サンプル.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Re05f306aec3e463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="Rc403fd97942b45c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R5a91f56d5cb84a25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="R8d73821883934440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R22f3b8dabb044c9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="Rfcc00a6be2dd416a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="R73c5ecd6c8a045f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="R28297a060f8343e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="R7d008b78fa2d46d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R1f5e7957ebf5412a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R614cff841ad246a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R61079fcad7844d41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="R94ab07ed12664ce5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="R81275d3652fe4f02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="R1326e5bd1a004d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="R976f9884f35d4771"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_担任授業期間ルール" sheetId="17" r:id="R96a728fc8ac1489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_操作説明" sheetId="1" r:id="Rde38277660b24c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_基本設定" sheetId="2" r:id="R97b63a58831b4598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_開講カレンダー" sheetId="3" r:id="R29738a44fbae4077"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_時限" sheetId="4" r:id="Rbf34e4f78a324312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_校舎" sheetId="5" r:id="R901d11ff3a6b4fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_教室" sheetId="6" r:id="Ra7eac23eed2b426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_教師" sheetId="7" r:id="Rb143050efc9e4416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_クラス" sheetId="8" r:id="Rcf9fc10571f24a1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_教科" sheetId="9" r:id="Ra5c75785d6a04789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_授業要求" sheetId="10" r:id="R6682dde8120646b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_教師休み" sheetId="11" r:id="R31d55cbc784c4b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_配置ルール" sheetId="12" r:id="R5995e1b8b2044e3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_選好設定" sheetId="13" r:id="Rea1ae067aaab4e07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_授業配置数ルール" sheetId="14" r:id="R03bd00b23dcc4a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_授業配置数選好ルール" sheetId="15" r:id="Rb7d7a31fe80641e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_教師休日日数ルール" sheetId="16" r:id="R662040bd0b784e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_担任授業期間ルール" sheetId="17" r:id="R168243d9056d4ae1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4253,7 +4253,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73a05fa7333740ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7f79643fc0b4bc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5349,7 +5349,7 @@
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="62" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
@@ -5371,32 +5371,30 @@
         <x:v>enabled</x:v>
       </x:c>
       <x:c r="D1" t="str">
-        <x:v>start_date</x:v>
+        <x:v>eligible_dates</x:v>
       </x:c>
       <x:c r="E1" t="str">
-        <x:v>end_date</x:v>
+        <x:v>required_days_off</x:v>
       </x:c>
       <x:c r="F1" t="str">
-        <x:v>required_days_off</x:v>
+        <x:v>minimum_days_off</x:v>
       </x:c>
       <x:c r="G1" t="str">
-        <x:v>minimum_days_off</x:v>
+        <x:v>maximum_days_off</x:v>
       </x:c>
       <x:c r="H1" t="str">
-        <x:v>maximum_days_off</x:v>
+        <x:v>preferred_days_off</x:v>
       </x:c>
       <x:c r="I1" t="str">
-        <x:v>preferred_days_off</x:v>
+        <x:v>quota_group_id</x:v>
       </x:c>
       <x:c r="J1" t="str">
-        <x:v>quota_group_id</x:v>
+        <x:v>group_required_days_off</x:v>
       </x:c>
       <x:c r="K1" t="str">
-        <x:v>group_required_days_off</x:v>
-      </x:c>
-      <x:c r="L1" t="str">
         <x:v>note</x:v>
       </x:c>
+      <x:c r="L1"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6571,7 +6569,7 @@
         <x:v>schema_version</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>0.9</x:v>
+        <x:v>1.0</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>入力契約バージョン</x:v>

</xml_diff>